<commit_message>
normalise layer abbreviations at index time; revert query-side expansion
</commit_message>
<xml_diff>
--- a/eval/RBI_NBFC_Retrieval_Questions_results.xlsx
+++ b/eval/RBI_NBFC_Retrieval_Questions_results.xlsx
@@ -512,12 +512,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The asset-size threshold for a non-deposit-taking NBFC-ICC to be classified in the Middle Layer is ₹1,000 crore. This is explicitly stated in the Middle Layer definition, which includes "non-deposit taking NBFCs with asset size of ₹1,000 crore and above" [3]. Consolidated group assets exceeding ₹1,000 crore may also place NBFC-ICC in the Middle Layer, but the general standalone threshold is ₹1,000 crore [1].</t>
+          <t>The asset-size threshold for a non-deposit-taking NBFC-ICC to be classified in the Middle Layer is ₹1,000 crore. This is explicitly stated in the Middle Layer definition, which includes "non-deposit taking NBFCs with asset size of ₹1,000 crore and above" [3]. Additionally, if consolidated group assets exceed ₹1,000 crore, NBFC-ICC may also be classified in the Middle Layer, but the general standalone threshold remains ₹1,000 crore [1].</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>8.199999999999999</v>
+        <v>12.1</v>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
@@ -566,7 +566,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under the 2025 NOF transition schedule, an existing NBFC-ICC must achieve a minimum Net Owned Fund (NOF) of ₹5 crore by March 31, 2025 [1].</t>
+          <t>Under the 2025 NOF transition schedule, an existing NBFC-ICC must achieve a minimum net owned fund (NOF) of ₹5 crore by March 31, 2025 [1].</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>8.300000000000001</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
@@ -620,12 +620,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The minimum CRAR for a Middle Layer NBFC-ICC is 15% of aggregate RWAs, and the minimum Tier 1 capital ratio is 10% of aggregate RWAs [2]. These requirements apply to NBFC-ML and above, including NBFC-ICC, as specified in the regulatory capital framework.</t>
+          <t>The minimum CRAR for a Middle Layer NBFC-ICC is 15% of aggregate RWAs, and the minimum Tier 1 capital ratio is 10% of aggregate RWAs [1]. These requirements apply as NBFC-ICC falls under the NBFC-Middle Layer category and is not primarily engaged in gold lending, which would trigger different thresholds [1][5].</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12944_Declaration-of-Dividends.pdf p.5 | 12953_Concentration-Risk-Management.pdf p.2</t>
+          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.2 | 12944_Declaration-of-Dividends.pdf p.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>7.6</v>
+        <v>9.5</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -674,12 +674,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The minimum Common Equity Tier 1 (CET1) ratio for an Upper Layer NBFC-ICC is 9 per cent of the aggregate RWAs, as specified for NBFC-UL in paragraph (4) of Chapter II Regulatory capital [1].</t>
+          <t>The minimum Common Equity Tier 1 (CET1) ratio for an Upper Layer NBFC-ICC is 9 per cent of the aggregate RWAs, as specified for all NBFC-UL entities in paragraph (4) of Chapter II Regulatory capital [1].</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2 | 12944_Declaration-of-Dividends.pdf p.6 | 13586_SUP-Miscellaneous.pdf p.8 | 12953_Concentration-Risk-Management.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21</t>
+          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2 | 12953_Concentration-Risk-Management.pdf p.10 | 12944_Declaration-of-Dividends.pdf p.6 | 13587_SUP-Supervisory-Returns.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.14</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>12.3</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -728,26 +728,26 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>The provided context passages do not specify the maximum leverage ratio for a Base Layer NBFC-ICC. The documents outline prudential requirements and applicability rules for various NBFC categories but do not explicitly state leverage ratio limits for Base Layer NBFC-ICCs.</t>
+          <t>The maximum leverage ratio for a Base Layer NBFC-ICC is seven, as specified in [3].</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.2 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.2 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.2 | 12947_Resolution-of-Stressed-Assets.pdf p.5</t>
+          <t>12953_Concentration-Risk-Management.pdf p.2 | 12931_Miscellaneous.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.20 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.2 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12947_Resolution-of-Stressed-Assets.pdf p.5</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>declined to answer an in-scope question - retrieval likely missed</t>
+          <t>no numeric facts to compare - read the answer yourself</t>
         </is>
       </c>
       <c r="J6" t="n">
-        <v>10.5</v>
+        <v>8.6</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -783,10 +783,10 @@
       <c r="F7" t="inlineStr">
         <is>
           <t>The standard periodic KYC update intervals are:  
-- **High-risk customers**: Once every **2 years** [1].  
-- **Medium-risk customers**: Once every **8 years** [1].  
-- **Low-risk customers**: Once every **10 years** [1].  
-These intervals apply from the date of account opening or the last KYC updation.</t>
+- **High-risk customers**: Every **2 years** [1].  
+- **Medium-risk customers**: Every **8 years** [1].  
+- **Low-risk customers**: Every **10 years** [1].  
+These intervals apply from the date of account opening or the last KYC updation. Low-risk individual customers may have an extended deadline until June 30, 2026, if applicable [1].</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -840,7 +840,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under the KYC directions, transaction records must be retained for **at least five years from the date of the transaction** [3]. Customer identification records, including details obtained during account opening and throughout the business relationship, must be preserved for **at least five years after the business relationship has ended** [3].</t>
+          <t>Under the KYC directions, transaction records must be retained for at least five years from the date of the transaction [3]. Customer identification and address records must be preserved for five years after the business relationship with the customer has ended [3].</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>5.8</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
@@ -894,12 +894,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>For an ordinary term loan at a Middle Layer NBFC-ICC, the overdue period triggering NPA classification is **more than 90 days**. This is specified in paragraph 51 of the context [2], which applies to NBFC-ML (Middle Layer NBFCs). Additionally, context [3] confirms that NBFC-ICC (including those with asset size ≥ ₹500 crore) follow the 90-day overdue threshold for NPA classification.</t>
+          <t>For an ordinary term loan at a Middle Layer NBFC-ICC, the overdue period triggering NPA classification is **more than 90 days**, as specified for NBFCs with asset size of ₹500 crore and above (including NBFC-ICC with CoR) under paragraph 45 of [3]. This applies because the glide path reduces the NPA threshold from 180 days to 90 days for such entities [3].</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12951_Securitisation-Transactions.pdf p.46</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.12</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -913,7 +913,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>8.6</v>
+        <v>11.7</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
@@ -948,12 +948,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The standard-asset provision for ordinary loans of a Middle Layer NBFC-ICC, excluding exposures with special provisioning rules, is **0.40 per cent** of the outstanding amount. This rate applies to NBFC-ML (Middle Layer) as specified in paragraph 55 of the context [4].</t>
+          <t>The standard-asset provision for ordinary loans of a Middle Layer NBFC-ICC, excluding exposures with special provisioning rules, is 0.40 per cent of the outstanding amount. This is specified in paragraph 55 of the provisioning requirements for NBFC-ML [1].</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.22 | 12953_Concentration-Risk-Management.pdf p.2 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.10 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.21 | 12931_Miscellaneous.pdf p.2 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.1 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.10 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.22 | 12933_Microfinance-Institution.pdf p.10</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -967,7 +967,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>10.9</v>
+        <v>11.6</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -1002,12 +1002,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under the 2025 transition schedule, NBFCs with overdue periods of more than 120 days must move to the 90-day NPA norm by **March 31, 2025** [1]. This is specified in the glide path outlined in paragraph 44 of the Reserve Bank of India (Non-Banking Financial Companies - Income Recognition, Asset Classification and Provisioning) Directions, 2025.</t>
+          <t>Under the 2025 transition schedule, a Base Layer NBFC must move from the 120-day to the 90-day NPA norm by **March 31, 2025**. This is specified in the glide path outlined in paragraph 44 of passage [1], which states that NBFCs with overdue periods of **more than 120 days** must transition to the 90-day NPA norm by March 31, 2025.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12949_Asset-Liability-Management.pdf p.10 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.28</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12961_Undertaking-of-Financial-Services.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12949_Asset-Liability-Management.pdf p.10 | 12947_Resolution-of-Stressed-Assets.pdf p.15</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>13.3</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The provided context passages do not specify the minimum and maximum public-deposit tenors applicable to an eligible deposit-taking NBFC-ICC. The regulations referenced focus on limits on deposit amounts, credit ratings, subscription norms, and compliance requirements, but none address the duration (tenor) of public deposits for NBFC-ICC.</t>
+          <t>The provided context passages do not specify the minimum and maximum public-deposit tenors applicable to an eligible deposit-taking NBFC-ICC. The discussions in the passages focus on limits on deposit amounts [1], subscription norms for NCDs [2], credit ratings [3], applicability of concentration risk management [4], auditor reporting requirements [5], and definitions [6], but none address the duration (tenor) of public deposits for NBFC-ICC.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1075,7 +1075,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>9.199999999999999</v>
+        <v>11.5</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
@@ -1110,7 +1110,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The public-deposit ceiling for an eligible NBFC-ICC meeting the minimum NOF and prudential requirements is **one and one-half times its NOF** [1]. For NBFC-ICC, the minimum NOF is ₹10 crore [2], so the ceiling would be **₹15 crore** (1.5 × ₹10 crore). This limit applies to accepting or renewing public deposits, with exceptions for matured deposits requiring depositor consent [1].</t>
+          <t>The public-deposit ceiling for an eligible NBFC-ICC meeting the minimum NOF and prudential requirements is **one and one-half times its NOF**. This is specified in [1], which states that such an NBFC shall not accept or renew public deposits exceeding 1.5 times its NOF.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1120,16 +1120,16 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>none of the expected figures appear (1.5times)</t>
+          <t>all key figures present (1.5times)</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>19.1</v>
+        <v>8.4</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1164,7 +1164,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>The context passages mention that NBFCs must obtain "minimum investment grade for fixed deposits" from an approved credit rating agency [1], but they do not specify the exact credit rating grade (e.g., AAA, AA, etc.). The term "minimum investment grade" is used generically without defining the precise rating level. Thus, the passages do not provide the exact minimum investment-grade credit rating prescribed.</t>
+          <t>The minimum investment-grade credit rating prescribed for public-deposit acceptance is "minimum investment grade" as specified in the Reserve Bank of India (Non-Banking Financial Companies - Acceptance of Public Deposits) Directions, 2025. This requirement is explicitly mentioned in paragraphs 12 and 13 of the Directions [1], and further referenced in the auditor's report obligations [2]. No specific rating symbol (e.g., AAA, AA) is provided in the passages.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1174,16 +1174,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>declined to answer an in-scope question - retrieval likely missed</t>
+          <t>no numeric facts to compare - read the answer yourself</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>5.7</v>
+        <v>5.9</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
@@ -1218,7 +1218,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Outside the hours of 8:00 a.m. to 7:00 p.m., recovery calls are prohibited for overdue loans other than microfinance loans. This is explicitly stated in [1], which prohibits calling borrowers before 8:00 a.m. or after 7:00 p.m. Additionally, [4] and [6] specify telephonic contact between 09:30 hours and 19:00 hours, but the stricter prohibition from [1] applies to recovery calls.</t>
+          <t>Recovery calls for overdue loans other than microfinance loans are prohibited outside the hours of 8:00 a.m. to 7:00 p.m. [1] (point 100). This restriction explicitly excludes microfinance loans under Reserve Bank of India directions [1]. Additionally, telemarketing contacts are generally restricted to 09:30 hours to 19:00 hours [4][6], but the specific prohibition for recovery calls applies to the 8:00 a.m.–7:00 p.m. window.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1237,7 +1237,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>16.8</v>
+        <v>12.8</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -1272,7 +1272,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>The minimum KFS validity period for retail and MSME term loans is **three working days** for loans with a tenor of seven days or more, and **one working day** for loans with a tenor of less than seven days [1].</t>
+          <t>The minimum KFS validity period for retail and MSME term loans is **three working days** for loans with a tenor of **seven days or more**. For loans with a tenor of **less than seven days**, the validity period is **one working day** [1].</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1291,7 +1291,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>8.699999999999999</v>
+        <v>7.4</v>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -1326,12 +1326,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A Middle Layer NBFC-ICC must appoint a Chief Risk Officer (CRO) if its asset size exceeds ₹5,000 crore. This is specified in [1], which mandates that NBFCs with assets over ₹5,000 crore appoint a CRO, regardless of their layer classification. The Middle Layer threshold (₹1,000 crore) [4] does not override this requirement.</t>
+          <t>A Middle Layer NBFC-ICC must appoint a Chief Risk Officer (CRO) if its asset size exceeds ₹5,000 crore. This is specified in [1], which states that NBFCs with asset size of more than ₹5,000 crore must appoint a CRO, regardless of their classification in the Middle Layer. The Middle Layer threshold (₹1,000 crore) is separate from the CRO requirement.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13588_SUP-Statutory-Audit.pdf p.7</t>
+          <t>12960_Governance.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 13588_SUP-Statutory-Audit.pdf p.7</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>10.1</v>
+        <v>7.3</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1380,12 +1380,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>A Middle Layer NBFC must submit its quarterly director-change statement and fit-and-proper certificate to the RBI's Regional Office within 15 days of the close of each quarter. The statement for the quarter ending March 31 must be certified by the auditors [1].</t>
+          <t>A Middle Layer NBFC must submit its quarterly director-change statement and fit-and-proper certificate to the Regional Office of the RBI's Department of Supervision within **15 days of the close of the respective quarter** [1]. The statement for the quarter ending March 31 must also be **certified by the auditors** [1].</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.9 | 12934_Peer-to-Peer-Lending-Platform.pdf p.17 | 12936_Account-Aggregator.pdf p.20 | 12953_Concentration-Risk-Management.pdf p.2 | 12960_Governance.pdf p.29 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
+          <t>12960_Governance.pdf p.9 | 12934_Peer-to-Peer-Lending-Platform.pdf p.17 | 12953_Concentration-Risk-Management.pdf p.2 | 12936_Account-Aggregator.pdf p.20 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12944_Declaration-of-Dividends.pdf p.6</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1399,7 +1399,7 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>10.3</v>
+        <v>8.9</v>
       </c>
       <c r="K18" t="inlineStr"/>
       <c r="L18" t="inlineStr"/>
@@ -1435,7 +1435,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>The reference dates for routine credit-bureau reporting under the November 28, 2025 version are the 9th, 16th, 23rd, and last day of the month [1]. For the full file submission, the deadline is the 5th day of the next month [1]. Incremental accounts for submissions on the 9th, 16th, and 23rd must be reported within four calendar days of those dates [1].</t>
+          <t>Under the November 28, 2025 version, routine credit-bureau reporting required submission of credit information on the 9th, 16th, 23rd, and last day of the month as reference dates [1]. For full-file submissions (containing all active and closed accounts as of the last day of the month), the deadline was the 5th day of the following month [1]. Incremental accounts for submissions on the 9th, 16th, and 23rd days must be reported within four calendar days of those dates [1].</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1454,7 +1454,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>9.1</v>
+        <v>6.7</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -1489,7 +1489,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The minimum cooling-off period for a digital loan is one day, as stipulated in [1]. The borrower must be given an explicit option to exit the loan during this period without penalty, and the NBFC determines the duration, which cannot be less than one day.</t>
+          <t>The minimum cooling-off period for a digital loan is one day, as stipulated in [1], which states that the NBFC must set the cooling-off period per their credit policy, subject to it not being less than one day.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1508,7 +1508,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>7.4</v>
+        <v>7.2</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
@@ -1543,7 +1543,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The percentage cap applicable to default loss guarantee (DLG) cover on an eligible digital-lending portfolio is **five per cent** of the total amount disbursed out of that loan portfolio at any given time. This is stipulated in the Cap on DLG provisions, which require NBFCs to ensure DLG cover does not exceed this threshold [2]. Additionally, the Default Loss Guarantee provisions explicitly state that originating NBFCs may provide such guarantees up to five per cent of loans outstanding in respect of loans under CLA [6].</t>
+          <t>The percentage cap applicable to default loss guarantee (DLG) cover on an eligible digital-lending portfolio is **five per cent** of the total amount disbursed from that loan portfolio at any given time. This is stipulated in the Cap on DLG provisions [2], which require NBFCs to ensure DLG cover does not exceed 5% of the disbursed amount. Additionally, this cap is referenced in provisions related to DLG arrangements under the Reserve Bank of India (Non-Banking Financial Companies - Credit Facilities) Directions, 2025 [5].</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1553,16 +1553,16 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>none of the expected figures appear (5%)</t>
+          <t>all key figures present (5%)</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
@@ -1597,12 +1597,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>The Base Layer (NBFCs-BL) consists of smaller NBFCs with lower risk profiles and a materiality threshold of ₹1 crore for loans [2]. The Middle Layer (NBFCs-ML) includes medium-sized NBFCs with a threshold of ₹5 crore [2], while the Upper Layer (NBFCs-UL) comprises larger NBFCs with a threshold of ₹10 crore [2]. The Top Layer (NBFCs-TL) is ideally empty but would presumably apply to the largest NBFCs, though no specific details are provided in the passages [1]. Regulatory requirements escalate with layer designation, with Upper Layer NBFCs subject to the most stringent rules [5].</t>
+          <t>The Base, Middle, Upper, and Top Layers categorize Non-Banking Financial Companies (NBFCs) based on size, activity, and risk, with distinct regulatory and operational requirements:  
+- **Base Layer (NBFCs-BL)**: NBFCs with smaller size and lower risk, such as NBFC-P2P, NBFC-AA, NOFHC, and Type I NBFCs [3]. Materiality thresholds for loans are ₹1 crore [2]. Regulatory compliance includes Chapter III only [5].  
+- **Middle Layer (NBFCs-ML)**: NBFCs with moderate size/risk, including HFCs, IFCs, SPD, and IDF-NBFCs [3]. Materiality thresholds are ₹5 crore [2]. Regulatory compliance includes Chapters II, III, and IV [5]. Governance requires EWS frameworks [6].  
+- **Upper Layer (NBFCs-UL)**: Larger, higher-risk NBFCs (e.g., NBFC-D, CIC, NBFC-IFC) with materiality thresholds of ₹10 crore [2]. Regulatory compliance includes Chapters II, III, IV, and V [5]. Governance mandates EWS frameworks and stricter oversight [6].  
+- **Top Layer (NBFCs-TL)**: Ideally empty, but if populated, would represent the highest-risk NBFCs with the strictest regulations [1].  
+Layer classification depends on asset size, activity, and supervisory assessments [4].</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12954_Credit-Risk-Management.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12937_Core-Investment-Companies.pdf p.6 | 12960_Governance.pdf p.3 | 12939_Housing-Finance-Companies.pdf p.6</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12954_Credit-Risk-Management.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12960_Governance.pdf p.3 | 13590_SUP-Fraud-Risk-Management.pdf p.10</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1616,7 +1621,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>6.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -1651,7 +1656,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Not taking customer deposits does not automatically mean an NBFC does not use public funds. According to [1], 'public funds' include not only public deposits but also inter-corporate deposits, bank finance, and funds from other sources like Commercial Papers or debentures. Thus, an NBFC could still use public funds through these alternative channels even if it does not accept customer deposits.</t>
+          <t>Not taking customer deposits does not necessarily mean an NBFC does not use public funds. According to [1], 'public funds' include funds raised through public deposits, inter-corporate deposits, bank finance, and other sources like Commercial Papers or debentures [18]. Thus, even if an NBFC avoids customer deposits (public deposits), it could still use other forms of public funds. The distinction hinges on whether the NBFC accepts any of these broader categories of public funds.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1670,7 +1675,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>5.9</v>
+        <v>6.5</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -1705,7 +1710,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>No, once a customer's KYC documents are checked, ongoing monitoring of transactions is required. The NBFC must conduct periodic KYC updation based on risk categories: high-risk customers require updates every 2 years, medium-risk every 8 years, and low-risk every 10 years [6]. Additionally, accounts opened via OTP-based e-KYC must undergo identification via V-CIP or CDD procedures within 1 year, otherwise operations are suspended [4]. The NBFC must also monitor for ML/TF activities and ensure compliance with periodic updation requirements, including advance notices and reminders to customers [5]. Thus, transaction monitoring cannot be discontinued after initial KYC verification.</t>
+          <t>No, once a customer's KYC documents are checked, monitoring of their transactions cannot be stopped. The NBFC must ensure periodic updation of KYC data, with intervals based on risk categories: high-risk customers require updates every 2 years, medium-risk every 8 years, and low-risk every 10 years [6]. Additionally, accounts opened via OTP-based e-KYC must undergo CDD within 1 year; otherwise, operations are suspended [4]. Failure to comply with periodic KYC updates may result in temporary cessation of account operations [5]. Thus, ongoing monitoring and verification are mandated.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1724,7 +1729,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>8.4</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1778,7 +1783,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>5</v>
+        <v>5.7</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1813,7 +1818,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>No, sending every borrower an English-only loan letter is not sufficient. The passages mandate that communications, including loan terms and conditions, must be in the vernacular language or a language as understood by the borrower [1], [2], [3]. For illiterate borrowers, important terms must be explained in the presence of a witness, regardless of language [3]. English-only communication would violate these requirements unless the borrower specifically understands English.</t>
+          <t>No, sending every borrower an English-only loan letter is not sufficient. The passages mandate that communications with borrowers must be in the vernacular language or a language as understood by the borrower [1], [2], [3]. For illiterate borrowers, terms and conditions must be explained in the presence of a witness, and all critical documents, including loan agreements and Key Fact Statements (KFS), must be in the language of the region or the language chosen by the borrower [3], [4]. English-only communication would violate these requirements unless the borrower explicitly understands English.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1832,7 +1837,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>5.3</v>
+        <v>5.9</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -1867,7 +1872,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Yes, borrowers must receive copies of all enclosures quoted in the loan agreement. According to the regulations, an NBFC shall "furnish a copy of the loan agreement along with a copy each of all enclosures quoted in the loan agreement to all the borrowers at the time of sanction/disbursement of loans" [1]. This requirement is reiterated in [2] and [3], which emphasize that such copies are necessary to ensure transparency and prevent disputes over terms and conditions.</t>
+          <t>Yes, borrowers must receive copies of all enclosures quoted in the loan agreement. According to the regulations, an NBFC shall "furnish a copy of the loan agreement along with a copy each of all enclosures quoted in the loan agreement to all the borrowers at the time of sanction/disbursement of loans" [1]. This requirement is reiterated in [2] and [3], emphasizing that such copies are necessary to ensure transparency and prevent disputes over terms and conditions.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1886,7 +1891,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1921,7 +1926,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>The Board of an NBFC should decide how to set lending rates, considering factors such as cost of funds, margin, and risk premium [1]. This is explicitly stated in paragraph 22 of the Responsible-Business-Conduct Directions, 2025, which mandates the Board to adopt an interest rate model incorporating these elements [1]. Additionally, paragraph 14 of the Housing-Finance-Companies Directions, 2026, reinforces this requirement, specifying that the interest rate model must account for these factors [3]. For microfinance loans, the Board must also approve a policy detailing the components of the interest rate, including cost of funds, risk premium, and margin, along with their quantum based on objective parameters [5].</t>
+          <t>The Board of an NBFC or HFC should decide how to set lending rates, considering factors such as cost of funds, margin, and risk premium [1], [3], [5]. They must also account for the nature of services provided, quantum of loans, and other objective parameters [5]. Additionally, they must ensure transparency by disclosing these factors to borrowers and aligning with regulatory norms and the Fair Practices Code [1], [4].</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1940,7 +1945,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>5.7</v>
+        <v>5.5</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1975,7 +1980,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Yes, the Board of an NBFC must disclose the rationale for charging different interest rates to different categories of borrowers. The rate of interest and the approach for gradations of risk must be explicitly communicated in the application form and the sanction letter, ensuring borrowers understand the basis for differential rates [1].</t>
+          <t>Yes, the Board of an NBFC must disclose the rationale for charging different interest rates to different categories of borrowers. The rate of interest and the approach for gradations of risk must be explicitly communicated in the sanction letter and application form, explaining the basis for differential rates [1].</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1994,7 +1999,7 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>5</v>
+        <v>5.2</v>
       </c>
       <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr"/>
@@ -2029,7 +2034,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>No, it is not solely the agency's problem. The Housing Finance Companies (HFCs) and Non-Banking Financial Companies (NBFCs) are legally obligated to ensure their recovery agents adhere to strict conduct guidelines, including prohibiting intimidation, harassment, and unlawful practices. For instance, HFCs must ensure contracts with recovery agents do not incentivize uncivilized behavior [1], and NBFCs are liable for their agents' actions, including ensuring they do not resort to harassment or false representations [2]. Additionally, HFCs must address grievances against their agents and cannot forward cases to recovery agencies until complaints are resolved [5]. Thus, the responsibility extends to the HFC/NBFC that engaged the agency.</t>
+          <t>No, it is not solely the agency's problem. The HFC/NBFC retains responsibility for ensuring recovery agents adhere to legal and ethical standards. For instance, HFCs must ensure contracts with recovery agents do not incentivize uncivilized behavior [1], and NBFCs are liable for their agents' actions, including harassment or intimidation [2]. Additionally, HFCs must address borrower grievances before involving recovery agents [5], and NBFCs must ensure agents comply with fair practices codes [4]. Thus, the HFC/NBFC shares accountability for the agency's conduct.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2048,7 +2053,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>7.4</v>
+        <v>7.1</v>
       </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -2083,7 +2088,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>No, the RBI does not require prior approval for an NBFC to enter into a financial-services outsourcing contract. According to [1], an NBFC "shall not require prior approval from RBI" for outsourcing financial services. However, such arrangements are subject to "on-site / offsite monitoring and inspection / scrutiny by RBI." Thus, approval is not a prerequisite for signing, but ongoing oversight is mandated.</t>
+          <t>No, an NBFC does not require prior approval from RBI to outsource financial services. The RBI does not mandate approval for such contracts, but the arrangements are subject to on-site/offsite monitoring and inspection by RBI [1].</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2102,7 +2107,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>5.2</v>
+        <v>4.7</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -2137,7 +2142,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>No, a CI must submit credit information to all CICs, not just CIBIL. According to passage [1], a CI "shall submit data ... to all CICs" [1]. The guidelines explicitly require reporting to all CICs, not selective reporting to a single entity like CIBIL.</t>
+          <t>No, a CI must submit credit information to all CICs, not just CIBIL. According to [1], a CI "shall submit data on credit information of its borrowers [...] to all CICs." This obligation applies to all CICs, including CIBIL.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2156,7 +2161,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>6.1</v>
+        <v>5</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -2191,7 +2196,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>No, the prohibition explicitly states that no NBFC shall accept any public deposit repayable on demand [1]. This prevents customers from demanding repayment at any time, unlike savings accounts. Premature repayment is allowed only after three months under specific conditions [4], but not on demand.</t>
+          <t>No, the prohibition in [1] explicitly states that NBFCs cannot accept public deposits repayable on demand. Additionally, [4] allows premature repayment only after three months from the deposit date, which is not equivalent to on-demand access. Thus, the product cannot function like a savings account with immediate repayment flexibility.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2210,7 +2215,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>5.5</v>
+        <v>5.8</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2245,7 +2250,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>No, for an ordinary loan that has become a Non-Performing Asset (NPA), unpaid interest cannot be booked as income. Income, including interest on NPAs, shall be recognized only when actually realized. Any income recognized before the asset became NPA and remaining unrealized shall be reversed [2] paragraph 38.</t>
+          <t>For an ordinary loan that has become a Non-Performing Asset (NPA), **unpaid interest cannot be booked as income**. Income recognition for NPAs is restricted to when it is *actually realised*. Any income recognised before the asset became non-performing and remaining unrealised must be reversed [2]§38. This applies regardless of the loan type, unless specific exceptions (e.g., moratorium periods) apply [2]§40.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2264,7 +2269,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>5.5</v>
+        <v>7.2</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2299,26 +2304,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Yes, a Middle Layer NBFC must appoint a Chief Compliance Officer (CCO). This is explicitly required under paragraph 1(1) of Chapter-II, which mandates Board-approved policies for "fit and proper" director status, CCO role definition, compensation policies, and Board reviews [1]. Additionally, paragraph 6 of the Governance document specifically states that Middle Layer NBFCs must appoint a CCO as part of ensuring an effective compliance culture [6]. The CCO's role includes promoting compliance culture, monitoring adherence to laws, and reporting directly to the Board or Managing Director [4].</t>
+          <t>The provided context passages do not mention whether a Middle Layer NBFC requires a designated compliance head. The discussions focus on regulatory layers, fraud risk management committees, and compliance with specific chapters of governance directions, but none explicitly address the need for a compliance head.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.7 | 12960_Governance.pdf p.29 | 13590_SUP-Fraud-Risk-Management.pdf p.7 | 13593_SUP-Compliance-Function.pdf p.10 | 13593_SUP-Compliance-Function.pdf p.7 | 12960_Governance.pdf p.12</t>
+          <t>12953_Concentration-Risk-Management.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 12960_Governance.pdf p.3 | 13590_SUP-Fraud-Risk-Management.pdf p.7 | 13590_SUP-Fraud-Risk-Management.pdf p.10</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>no numeric facts to compare - read the answer yourself</t>
+          <t>declined to answer an in-scope question - retrieval likely missed</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>5.5</v>
+        <v>8.1</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -2353,7 +2358,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>The vendor's promise alone is not sufficient. The outsourcing agreement must include specific contingency plans to ensure testing requirements [1](x) and business continuity measures [2](f). Additionally, the agreement must detail resolution processes, indemnities, and remedial actions for outages, as outlined in [1](ix) and [2](e). These provisions require contractual mechanisms rather than mere promises.</t>
+          <t>The vendor's promise alone is not sufficient. The outsourcing agreement must include specific contingency plans to ensure testing requirements [1](x), business continuity measures [2](f), and provisions for risk mitigation strategies [4](15). Additionally, the agreement must grant the NBFC or HFC rights to audit the service provider [1](ii), access IT infrastructure [1](xii), and enforce termination clauses [2](d). These requirements are explicitly outlined in the regulatory frameworks, indicating that contractual clauses and documented safeguards, not mere promises, are necessary.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2372,7 +2377,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>7</v>
+        <v>7.5</v>
       </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -2407,12 +2412,12 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>If the consolidated assets of the group (₹600 crore + ₹500 crore = ₹1,100 crore) exceed ₹1,000 crore, the NBFC-ICCs must be classified in the Middle Layer per [1] §18. Standalone asset sizes alone determine Base Layer status [2], but group consolidation overrides this for classification purposes. Thus, both NBFC-ICCs cannot remain in the Base Layer.</t>
+          <t>No, the two NBFC-ICCs cannot both remain in the Base Layer. According to [1], if the consolidated asset size of NBFCs in a group reaches ₹1000 crore or more, all NBFCs in the group (including NBFC-ICC) are classified as Middle Layer. In this case, the consolidated assets of ₹600 crore + ₹500 crore = ₹1100 crore exceed the ₹1000 crore threshold, triggering Middle Layer classification for both NBFC-ICCs. [3] further clarifies that NBFC-ICC is by default in the Base Layer unless consolidation pushes them to Middle Layer. Thus, they must be classified in the Middle Layer.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.3 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12936_Account-Aggregator.pdf p.3 | 12953_Concentration-Risk-Management.pdf p.2</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.3 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2426,7 +2431,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>9.699999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2461,12 +2466,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>No, you cannot immediately stop Middle Layer reporting. According to [1], if an NBFC's asset size temporarily falls below ₹1,000 crore due to fluctuations, it must continue complying with Middle Layer reporting requirements and extant directions until the submission of its next audited balance sheet to the Reserve Bank and a specific dispensation from the RBI is obtained. The threshold for classification as NBFC-ML is based on the consolidated asset size [3], but temporary dips below ₹1,000 crore do not exempt the NBFC from ongoing obligations.</t>
+          <t>No, you cannot immediately stop Middle Layer reporting. According to [1], if an NBFC's asset size falls below ₹1,000 crore due to temporary fluctuations, it must continue complying with Middle Layer reporting requirements and extant directions until the submission of its next audited balance sheet to the Reserve Bank and a specific dispensation is granted. Temporary declines in asset size do not exempt NBFCs from ongoing obligations until formal reassessment by the RBI.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13587_SUP-Supervisory-Returns.pdf p.8 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13587_SUP-Supervisory-Returns.pdf p.8</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2480,7 +2485,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>6</v>
+        <v>6.6</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
@@ -2515,12 +2520,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>The NBFC is not capital-compliant. As a Middle Layer NBFC-ICC, it must maintain a minimum Tier 1 capital of 10% of aggregate RWAs [4]. The entity's Tier 1 capital is 9%, which is below the 10% regulatory minimum. While its CRAR of 17% exceeds the 15% requirement for NBFC-ML [4], the Tier 1 capital shortfall violates the Tier 1 capital adequacy rule. This places it in Tier 1 Capital Ratio Risk Threshold-1 (currently Tier 1 &lt;10% but ≥8%) [1], which is below the regulatory minimum.</t>
+          <t>The NBFC-ICC as a Middle Layer NBFC must maintain a minimum Tier 1 capital of 10% of aggregate RWAs [3]. With only 9% Tier 1 capital, it fails to meet this requirement. While its CRAR of 17% exceeds the 15% minimum for Middle Layer NBFCs [3], Tier 1 capital alone must meet the 10% threshold. Thus, the NBFC is not capital-compliant.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.10 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2</t>
+          <t>12953_Concentration-Risk-Management.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12944_Declaration-of-Dividends.pdf p.6 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 13586_SUP-Miscellaneous.pdf p.8</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2534,7 +2539,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -2569,7 +2574,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>No, you should not continue questioning the customer. If there is a suspicion of money laundering and performing further KYC checks would reasonably alert the customer, the NBFC is instructed to refrain from pursuing the CDD process and instead file an STR with FIU-IND [1].</t>
+          <t>If the NBFC forms a suspicion of money laundering or terrorist financing and reasonably believes that performing the CDD process will tip off the customer, it shall not pursue the CDD process and instead file an STR with FIU-IND [1]. Thus, in such circumstances, further KYC questioning should not continue.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2588,7 +2593,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>5.2</v>
+        <v>6.1</v>
       </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
@@ -2623,12 +2628,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>No, the loan cannot be upgraded to standard. According to paragraph 25 of [1], for borrowers with multiple credit facilities, loan accounts classified as NPA may be upgraded to standard only upon repayment of **entire arrears of interest and principal pertaining to all** credit facilities. Since the borrower has two loans (facilities) classified as NPA, clearing arrears on just one does not satisfy the requirement for upgradation. The entire arrears across all facilities must be repaid.</t>
+          <t>No, the loan cannot become standard. According to paragraph 25 of [1], loan accounts classified as NPA may be upgraded to standard only upon repayment of **entire arrears of interest and principal pertaining to all** credit facilities. Since the borrower has cleared arrears for only one of the two loans, the entire account (both loans) remains classified as NPA. Additionally, paragraph 24 of [1] specifies that an NPA can be upgraded to standard only if **entire arrears** (interest and principal) are paid, which is not satisfied here.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12957_Credit-Facilities.pdf p.29 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.24 | 12947_Resolution-of-Stressed-Assets.pdf p.35 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.26 | 12947_Resolution-of-Stressed-Assets.pdf p.52</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12947_Resolution-of-Stressed-Assets.pdf p.52 | 12957_Credit-Facilities.pdf p.29 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2642,7 +2647,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>6.7</v>
+        <v>7.9</v>
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
@@ -2677,7 +2682,12 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>The digital-lending partner's request to receive disbursements in its own pool account and then transfer them to borrowers is **not permitted**. According to context [2], paragraph 2, point (2): "Loan servicing, repayment, etc. is executed by the borrower directly in the NBFC's account without any pass-through account or pool account of any third party." This explicitly prohibits the use of third-party pool accounts for disbursements or servicing activities. Thus, funds must be transferred directly to the borrower's bank account, not through a pool account [2].</t>
+          <t>The digital-lending partner's request to receive disbursements in its own pool account and then transfer them to borrowers is **not permitted**. 
+Under the regulations, NBFC-P2P platforms are prohibited from holding funds received from lenders on their own balance sheet, including through pool accounts. Specifically:  
+- Funds from lenders must be transferred to the **Lenders' Escrow Account** and disbursed directly to the borrower's bank account **after compliance with paragraph 34** [1].  
+- The NBFC-P2P **cannot hold funds** for servicing loans or use pool accounts for this purpose, as this would violate the requirement that "funds received from lenders... shall not be held on its own balance sheet" [3].  
+- All fund transfers must occur **through and from bank accounts**, with **cash transactions strictly prohibited** [1].  
+Thus, the proposed mechanism involving a pool account would breach these prudential norms.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2696,7 +2706,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>8.4</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
@@ -2731,7 +2741,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>The NBFC's collection of data, including contact lists, must be need-based and with explicit consent, but accessing mobile phone resources like contact lists is explicitly prohibited [1]. While a consent checkbox may be part of the process, the regulation explicitly forbids accessing contact lists under any circumstances, even with consent. Thus, consent alone is insufficient to justify such access.</t>
+          <t>Consent alone is not sufficient. The NBFC must ensure that data collection is need-based, with prior and explicit consent, and that the consent artefact includes standardized details such as the purpose of data collection, recipients, and revocation rights [1][3]. Access to mobile resources like contact lists is explicitly prohibited unless for onboarding/KYC purposes [1]. Since credit scoring is not explicitly listed as a permitted purpose for contact list access, even with consent, the practice may violate regulations.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2750,7 +2760,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>7.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -2785,12 +2795,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>No, an NBFC cannot automatically increase credit limits for customers who repay on time. According to [1] §8(2), an NBFC must ensure there is no automatic increase in credit limits unless an explicit request is received, evaluated, and kept on record from the borrower. Automatic increases without such a request are prohibited.</t>
+          <t>No, an NBFC cannot automatically increase credit limits for customers who repay on time. According to [2](2), an NBFC shall ensure there is no automatic increase in credit limit unless an explicit request is received, evaluated, and kept on record from the borrower. Automatic adjustments without such a request are prohibited.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>12957_Credit-Facilities.pdf p.15 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.6 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.18 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.27 | 12947_Resolution-of-Stressed-Assets.pdf p.54 | 12942_Responsible-Business-Conduct.pdf p.18</t>
+          <t>13591_SUP-Digital-Payment-Security-Controls.pdf p.6 | 12957_Credit-Facilities.pdf p.15 | 12942_Responsible-Business-Conduct.pdf p.16 | 12942_Responsible-Business-Conduct.pdf p.18 | 12943_Know-Your-Customer.pdf p.40 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2804,7 +2814,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>6.9</v>
+        <v>5.7</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
@@ -2839,12 +2849,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>No, you cannot outsource the final decision to sanction retail loans to an unrelated fintech vendor. According to [1], NBFCs are prohibited from outsourcing core management functions, including "decision-making functions such as determining compliance with KYC norms for opening deposit accounts, giving sanction for loans (including retail loans)." This restriction applies regardless of whether the service provider is related or unrelated. While [4] allows NBFCs to engage lenders (LSPs) for digital lending, it explicitly states that the NBFC remains fully responsible for all acts and omissions of the LSP, including loan sanctioning decisions. Thus, the final sanctioning authority cannot be delegated to an external vendor.</t>
+          <t>The decision to sanction retail loans is explicitly listed as a core management function that **shall not be outsourced** [1]. This prohibition applies regardless of the NBFC's layer (including Middle Layer). While Middle Layer NBFCs are subject to specific outsourcing provisions [2], the sanctioning of loans (including retail loans) remains a non-outsourcable function. Thus, outsourcing this decision to an unrelated fintech vendor is not permitted.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>12941_Managing-Risks-in-Outsourcing.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12941_Managing-Risks-in-Outsourcing.pdf p.24 | 12957_Credit-Facilities.pdf p.14 | 12954_Credit-Risk-Management.pdf p.13 | 12941_Managing-Risks-in-Outsourcing.pdf p.37</t>
+          <t>12941_Managing-Risks-in-Outsourcing.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12941_Managing-Risks-in-Outsourcing.pdf p.24 | 12954_Credit-Risk-Management.pdf p.13 | 12957_Credit-Facilities.pdf p.14 | 12941_Managing-Risks-in-Outsourcing.pdf p.13</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2858,7 +2868,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>8.199999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
@@ -2893,7 +2903,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>No, a formal outsourcing agreement cannot be skipped. According to [1], NBFCs must have written agreements with group entities, including Service Level Agreements (SLAs), and [5] mandates that outsourcing agreements must be legally binding and include terms like access to records, confidentiality, and risk management. Additionally, [5] explicitly requires agreements to define rights and obligations, even for related parties. Skipping such an agreement would violate regulatory requirements for transparency, risk management, and accountability.</t>
+          <t>No, you cannot skip a formal outsourcing agreement. The context explicitly requires that even when outsourcing to a group entity (related party), the NBFC must ensure the arrangement is documented in a legally binding written agreement with detailed terms, including service scope, confidentiality, audit rights, and risk management provisions [1], [4], [5]. Additionally, the agreement must allow the NBFC to maintain control, ensure compliance with regulatory oversight (e.g., RBI inspections), and include clauses for termination and data protection [1], [4], [5]. Risk management practices for group entities are identical to those for non-related parties [1].</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2912,7 +2922,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>7.2</v>
+        <v>9.6</v>
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
@@ -2947,12 +2957,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>No, it is not allowed. Key Managerial Personnel (KMP) of an NBFC shall not hold any office (including directorships) in any other NBFC-ML or NBFC-UL except for directorships in NBFCs-BL [1]. Since the proposed directorship is in another Middle Layer NBFC (NBFC-ML), this violates the restriction.</t>
+          <t>No, it is not allowed. Key Managerial Personnel (KMP) of an NBFC in the Middle Layer (NBFC-ML) cannot hold directorships in other NBFC-ML or NBFC-UL entities unless the position is in a subsidiary. The CFO, as KMP, cannot assume directorship in another Middle Layer NBFC that is not a subsidiary [1].</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.12 | 12953_Concentration-Risk-Management.pdf p.2 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12960_Governance.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4</t>
+          <t>12960_Governance.pdf p.12 | 12960_Governance.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12944_Declaration-of-Dividends.pdf p.6 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 12961_Undertaking-of-Financial-Services.pdf p.2</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2966,7 +2976,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>6.6</v>
+        <v>7.4</v>
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
@@ -3001,7 +3011,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>No. If an NBFC's credit rating is downgraded below the minimum investment grade, it must immediately stop accepting fresh public deposits and renewing existing deposits [1]. The downgraded status triggers this cessation regardless of ongoing efforts to upgrade the rating. Existing deposits must run off to maturity, and the NBFC must report the situation to the Reserve Bank within fifteen working days [1].</t>
+          <t>No, the NBFC cannot renew existing public deposits if its credit rating has been downgraded below the minimum investment grade. According to [1], in such cases, the NBFC must immediately stop accepting fresh public deposits and renewing existing ones. Additionally, [2] states that if public deposits exceed one and one-half times the NOF, the NBFC cannot renew or accept fresh deposits until the limit is restored. Thus, during the downgraded period, renewals are prohibited.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3020,7 +3030,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>5.6</v>
+        <v>6.7</v>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -3055,11 +3065,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Adding a 2% penal interest rate after a missed EMI and compounding it is **not permitted**. 
-- Penal charges (including penal interest) **cannot be capitalized**, meaning no further interest can be computed on such charges [1]. 
-- While normal compounding of **unpaid interest** (at the contracted rate) is allowed until remediation, **penal charges themselves cannot be compounded** [1][3]. 
-- The 2% penal interest would be treated as a separate charge, and compounding it would violate the prohibition on capitalizing penal charges. 
-Thus, the proposed approach violates the guidelines.</t>
+          <t>Adding a 2% penal interest rate after a missed EMI is permitted, but compounding it is not allowed. Penal charges for non-compliance (e.g., missed EMI) must be treated as separate fees and **not capitalized** (i.e., no further interest computed on such charges) [1][3]. However, normal compounding of interest on unpaid interest (including unpaid EMI) at the contracted rate is allowed until remediation [1]. Thus, the 2% penal interest can be applied, but it cannot be compounded.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3078,7 +3084,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>9.5</v>
+        <v>7.2</v>
       </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -3113,12 +3119,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Yes, you must report the LSP's lending app to the RBI. According to [1](1), an NBFC must report all DLAs "deployed / joined by them," whether their own or those of LSPs, as a platform participant. This includes reporting DLAs of third parties (like the LSP's app) if the NBFC participates in deploying or joining them. The requirement applies regardless of ownership, as the NBFC is acting as a platform participant. The Chief Compliance Officer must certify the DLA's compliance with regulatory requirements, including linking to the NBFC's website and grievance mechanisms [1](4).</t>
+          <t>Yes, as a Middle Layer NBFC joining an LSP's lending app alongside other lenders, you must report the app to the RBI. According to [1] (18. Reporting of DLAs to RBI), an NBFC must report all DLAs "deployed / joined by them, whether their own or those of the LSPs" on the CIMS portal. This includes participating as a platform participant, even if the app is not owned by the NBFC. The requirement applies regardless of ownership, as the NBFC is actively involved in the arrangement.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>12957_Credit-Facilities.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.20 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12957_Credit-Facilities.pdf p.15</t>
+          <t>12957_Credit-Facilities.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12931_Miscellaneous.pdf p.2 | 12957_Credit-Facilities.pdf p.14 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12941_Managing-Risks-in-Outsourcing.pdf p.4</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3132,7 +3138,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>8.4</v>
+        <v>7.2</v>
       </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
@@ -3167,7 +3173,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>No. Changes in interest rates and charges must be effected prospectively, not retrospectively. According to [1], NBFCs must ensure changes in interest rates and charges are applied prospectively. Additionally, [6] explicitly states that no charges or fees can be levied retrospectively at the time of prepayment of loans. Thus, applying a higher contractual rate retrospectively from last month would violate these provisions.</t>
+          <t>No. According to [1], changes in interest rates and charges must be "effected only prospectively," meaning they cannot apply retrospectively. Additionally, [6](8) explicitly prohibits NBFCs from levying charges retrospectively, including pre-payment charges, unless disclosed in advance. Thus, notifying borrowers of a higher contractual rate applying from last month would violate these provisions.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -3186,7 +3192,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>8.199999999999999</v>
+        <v>7</v>
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
@@ -3220,7 +3226,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>The provided context passages do not contain information about SEBI rules governing minimum public shareholding or offer-allocation requirements for NBFCs planning an IPO. The passages focus on RBI regulations related to NBFC operations, such as sponsorship of mutual funds, investment norms, and concentration risk management, but none address SEBI's IPO-specific guidelines.</t>
+          <t>The provided context passages do not contain information about SEBI rules governing minimum public shareholding or offer-allocation requirements for NBFCs planning an IPO. The passages focus on RBI regulations related to NBFCs (e.g., sponsorship of IDF-MFs, concentration risk management, and investment guidelines), but none address SEBI's specific requirements for IPOs.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3239,7 +3245,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>7.6</v>
+        <v>7.4</v>
       </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
@@ -3292,7 +3298,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>6</v>
+        <v>6.1</v>
       </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
@@ -3326,7 +3332,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>The provided context passages do not contain information about insider-trading rules or trading window closure dates for listed NBFC employees.</t>
+          <t>The provided context passages do not contain information about insider-trading rules, trading windows, or specific deadlines for NBFC employees regarding quarterly results.</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -3345,7 +3351,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>5.9</v>
+        <v>5.7</v>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
@@ -3379,7 +3385,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>The context specifies that employees dealing with insurance agency/broking business must "possess the requisite qualification prescribed by IRDA" [1]. However, the passages do not detail the specific examinations, training programs, or certification requirements mandated by IRDA for these roles. The focus is on compliance with IRDA regulations rather than enumerating exact training modules or exams.</t>
+          <t>The context specifies that employees dealing with insurance agency/broking business must possess "the requisite qualification prescribed by IRDA" [1]. However, the passages do not explicitly name specific examinations or training programs required for these qualifications. The focus is on compliance with IRDA regulations rather than detailing particular exams or training courses.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3398,7 +3404,7 @@
         </is>
       </c>
       <c r="J55" t="n">
-        <v>6.7</v>
+        <v>7.8</v>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
@@ -3485,7 +3491,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>The context passages do not specify the GST rate applicable to loan-processing fees or the timing for issuing tax invoices. The only mention of GST relates to penal charges, requiring NBFCs to follow CBIC instructions [4], but no details are provided about loan-processing fees.</t>
+          <t>The provided context passages do not specify the GST rate applicable to loan-processing fees or the timing for issuing tax invoices. The only mention of GST relates to penal charges, stating that NBFCs must follow CBIC instructions on its applicability [4]. No details about GST rates or invoicing timelines for loan-processing fees are provided.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3504,7 +3510,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>7.2</v>
+        <v>7.3</v>
       </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
@@ -3538,7 +3544,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>The provided context passages do not address whether an NBFC can claim an income-tax deduction for provisions created against bad loans. The discussions focus on accounting disclosures, prudential norms, provisioning requirements, and asset classification, but none mention tax treatment or deductibility of such provisions.</t>
+          <t>The provided context passages do not address whether an NBFC can claim an income-tax deduction for provisions created against bad loans. The discussions focus on accounting disclosures, prudential norms, provisioning requirements, and asset classification, but none mention tax treatment or deductibility of provisions.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -3557,7 +3563,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>7.2</v>
+        <v>7.1</v>
       </c>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
@@ -3591,7 +3597,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>The provided context passages do not mention TDS rates, exemption thresholds, or any tax-related provisions applicable to interest payments on resident customers' fixed deposits.</t>
+          <t>The provided context passages do not mention TDS rates or exemption thresholds for interest payments on resident customers' fixed deposits. The documents focus on legal agreements, interest rate sensitivity statements, and deposit management procedures, but none address tax deduction at source (TDS) regulations or tax exemption thresholds. For this query, refer to the Income Tax Act, 1961, or relevant circulars from the Income Tax Department.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3610,7 +3616,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>6.5</v>
+        <v>8.6</v>
       </c>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
@@ -3644,7 +3650,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>The context passages do not specify the Companies Act filing deadlines for AOC-4 financial statements or MGT-7 annual returns.</t>
+          <t>The context passages do not specify the Companies Act filing deadlines for AOC-4 financial statements or MGT-7 annual returns. The provided information addresses timelines for other returns (e.g., DNBS10, Fraud Monitoring Returns) but does not mention AOC-4 or MGT-7 directly [1][4]. For precise deadlines, reference to the Companies Act, 2013, or relevant regulatory guidelines would be required.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -3663,7 +3669,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>7.7</v>
+        <v>8</v>
       </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
@@ -3697,7 +3703,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>The provided context passages do not contain information about calculating Companies Act CSR (Corporate Social Responsibility) spending obligations or transferring unspent CSR amounts.</t>
+          <t>The provided context passages do not contain information about calculating CSR (Corporate Social Responsibility) spending obligations under the Companies Act or transferring unspent CSR amounts. The passages focus on definitions related to public deposits, financial regulations, and capital adequacy, but none address CSR requirements or procedures.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -3716,7 +3722,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>5.7</v>
+        <v>6.6</v>
       </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>

</xml_diff>

<commit_message>
baseline before generated questions
</commit_message>
<xml_diff>
--- a/eval/RBI_NBFC_Retrieval_Questions_results.xlsx
+++ b/eval/RBI_NBFC_Retrieval_Questions_results.xlsx
@@ -512,12 +512,12 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>The asset-size threshold for a non-deposit-taking NBFC-ICC to be classified in the Middle Layer is ₹1,000 crore. This is explicitly stated in the Middle Layer definition, which includes "non-deposit taking NBFCs with asset size of ₹1,000 crore and above" [3]. Additionally, if consolidated group assets exceed ₹1,000 crore, NBFC-ICC may also be classified in the Middle Layer, but the general standalone threshold remains ₹1,000 crore [1].</t>
+          <t>The asset-size threshold for a non-deposit-taking NBFC-ICC to be classified in the Middle Layer is ₹1,000 crore. This is explicitly stated in [3], which defines the Middle Layer as including "non-deposit taking NBFCs with asset size of ₹1,000 crore and above." Additionally, [4] confirms that once an NBFC reaches this threshold, it is subject to Middle Layer regulatory requirements.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -531,7 +531,7 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>12.1</v>
+        <v>24.1</v>
       </c>
       <c r="K2" t="inlineStr"/>
       <c r="L2" t="inlineStr"/>
@@ -566,26 +566,26 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Under the 2025 NOF transition schedule, an existing NBFC-ICC must achieve a minimum net owned fund (NOF) of ₹5 crore by March 31, 2025 [1].</t>
+          <t>Under the 2025 NOF transition schedule, existing NBFC-ICC must achieve a minimum net owned fund (NOF) of ₹5 crore by March 31, 2025. This is specified in the glide path outlined in [1] (paragraph 42), which details the phased requirements for NBFC-ICC to reach ₹10 crore by March 31, 2027.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12939_Housing-Finance-Companies.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.6 | 12939_Housing-Finance-Companies.pdf p.8 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12953_Concentration-Risk-Management.pdf p.10</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12939_Housing-Finance-Companies.pdf p.13 | 12931_Miscellaneous.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.6 | 12939_Housing-Finance-Companies.pdf p.8 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>found 5crore, 31, 2025; missing 10crore, 2027.</t>
+          <t>all key figures present (5crore, 31, 2025, 10crore, 2027.)</t>
         </is>
       </c>
       <c r="J3" t="n">
-        <v>9.699999999999999</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K3" t="inlineStr"/>
       <c r="L3" t="inlineStr"/>
@@ -620,12 +620,12 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>The minimum CRAR for a Middle Layer NBFC-ICC is 15% of aggregate RWAs, and the minimum Tier 1 capital ratio is 10% of aggregate RWAs [1]. These requirements apply as NBFC-ICC falls under the NBFC-Middle Layer category and is not primarily engaged in gold lending, which would trigger different thresholds [1][5].</t>
+          <t>The minimum CRAR for a Middle Layer NBFC-ICC (not primarily a gold lender) is 15% of aggregate RWAs, and the minimum Tier 1 capital ratio is 10% of aggregate RWAs [2].</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.2 | 12944_Declaration-of-Dividends.pdf p.5</t>
+          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.10 | 12944_Declaration-of-Dividends.pdf p.5</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>9.5</v>
+        <v>6.7</v>
       </c>
       <c r="K4" t="inlineStr"/>
       <c r="L4" t="inlineStr"/>
@@ -674,12 +674,12 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>The minimum Common Equity Tier 1 (CET1) ratio for an Upper Layer NBFC-ICC is 9 per cent of the aggregate RWAs, as specified for all NBFC-UL entities in paragraph (4) of Chapter II Regulatory capital [1].</t>
+          <t>The minimum Common Equity Tier 1 (CET1) ratio for an Upper Layer NBFC-ICC is 9 per cent of the aggregate RWAs, as specified for NBFC-UL (Upper Layer) in paragraph (4) of Chapter II Regulatory capital [1].</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2 | 12953_Concentration-Risk-Management.pdf p.10 | 12944_Declaration-of-Dividends.pdf p.6 | 13587_SUP-Supervisory-Returns.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.14</t>
+          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.10 | 12944_Declaration-of-Dividends.pdf p.6 | 13586_SUP-Miscellaneous.pdf p.8 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -693,7 +693,7 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>8.300000000000001</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr"/>
@@ -728,12 +728,12 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>The maximum leverage ratio for a Base Layer NBFC-ICC is seven, as specified in [3].</t>
+          <t>The maximum leverage ratio for a Base Layer NBFC-ICC is seven, as specified in [3] for NBFC-BL (Base Layer). Since NBFC-ICC is classified under Base Layer, the same leverage ratio applies.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>12953_Concentration-Risk-Management.pdf p.2 | 12931_Miscellaneous.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.20 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.2 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12947_Resolution-of-Stressed-Assets.pdf p.5</t>
+          <t>12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.20 | 12931_Miscellaneous.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.2 | 12941_Managing-Risks-in-Outsourcing.pdf p.4</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -747,7 +747,7 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>8.6</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
@@ -782,16 +782,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>The standard periodic KYC update intervals are:  
-- **High-risk customers**: Every **2 years** [1].  
-- **Medium-risk customers**: Every **8 years** [1].  
-- **Low-risk customers**: Every **10 years** [1].  
-These intervals apply from the date of account opening or the last KYC updation. Low-risk individual customers may have an extended deadline until June 30, 2026, if applicable [1].</t>
+          <t>The standard periodic KYC update intervals are: high-risk customers every 2 years, medium-risk customers every 8 years, and low-risk customers every 10 years from the date of account opening or last KYC updation [1].</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>12943_Know-Your-Customer.pdf p.41 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.56 | 12943_Know-Your-Customer.pdf p.44 | 12943_Know-Your-Customer.pdf p.21 | 12943_Know-Your-Customer.pdf p.34</t>
+          <t>12943_Know-Your-Customer.pdf p.41 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.57 | 12943_Know-Your-Customer.pdf p.44 | 12943_Know-Your-Customer.pdf p.21 | 12943_Know-Your-Customer.pdf p.34</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -805,7 +801,7 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>6.8</v>
+        <v>6.1</v>
       </c>
       <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
@@ -840,12 +836,12 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Under the KYC directions, transaction records must be retained for at least five years from the date of the transaction [3]. Customer identification and address records must be preserved for five years after the business relationship with the customer has ended [3].</t>
+          <t>Under the KYC directions, transaction records must be retained for at least five years from the date of the transaction [3], and customer identification records, including addresses, must be preserved for five years after the business relationship with the customer ends [3].</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>12943_Know-Your-Customer.pdf p.34 | 12943_Know-Your-Customer.pdf p.56 | 12943_Know-Your-Customer.pdf p.48 | 12943_Know-Your-Customer.pdf p.41 | 12943_Know-Your-Customer.pdf p.44 | 12943_Know-Your-Customer.pdf p.15</t>
+          <t>12943_Know-Your-Customer.pdf p.34 | 12943_Know-Your-Customer.pdf p.57 | 12943_Know-Your-Customer.pdf p.48 | 12943_Know-Your-Customer.pdf p.41 | 12943_Know-Your-Customer.pdf p.6 | 12943_Know-Your-Customer.pdf p.44</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -859,7 +855,7 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>8.300000000000001</v>
+        <v>5.6</v>
       </c>
       <c r="K8" t="inlineStr"/>
       <c r="L8" t="inlineStr"/>
@@ -894,12 +890,12 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>For an ordinary term loan at a Middle Layer NBFC-ICC, the overdue period triggering NPA classification is **more than 90 days**, as specified for NBFCs with asset size of ₹500 crore and above (including NBFC-ICC with CoR) under paragraph 45 of [3]. This applies because the glide path reduces the NPA threshold from 180 days to 90 days for such entities [3].</t>
+          <t>For an ordinary term loan at a Middle Layer NBFC-ICC, the overdue period triggering NPA classification is **more than 90 days**, as specified in paragraph 44 of [3], which applies to NBFC-ICC with CoR under the Factoring Regulation Act, 2011. This aligns with the 90-day threshold for NPA classification for such entities.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.12</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12951_Securitisation-Transactions.pdf p.46</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -913,7 +909,7 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>11.7</v>
+        <v>22.7</v>
       </c>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
@@ -948,12 +944,12 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>The standard-asset provision for ordinary loans of a Middle Layer NBFC-ICC, excluding exposures with special provisioning rules, is 0.40 per cent of the outstanding amount. This is specified in paragraph 55 of the provisioning requirements for NBFC-ML [1].</t>
+          <t>The standard-asset provision for ordinary loans of a Middle Layer NBFC-ICC, excluding exposures with special provisioning rules, is 0.40 per cent of the outstanding amount [1].</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.1 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.10 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.22 | 12933_Microfinance-Institution.pdf p.10</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.22 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.10 | 12931_Miscellaneous.pdf p.2</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -967,7 +963,7 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>11.6</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="K10" t="inlineStr"/>
       <c r="L10" t="inlineStr"/>
@@ -1002,12 +998,12 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Under the 2025 transition schedule, a Base Layer NBFC must move from the 120-day to the 90-day NPA norm by **March 31, 2025**. This is specified in the glide path outlined in paragraph 44 of passage [1], which states that NBFCs with overdue periods of **more than 120 days** must transition to the 90-day NPA norm by March 31, 2025.</t>
+          <t>Under the 2025 transition schedule, a Base Layer NBFC must move from the 120-day to the 90-day NPA norm by **March 31, 2025**. This is specified in the glide path outlined in paragraph 44 of [1], which states that NBFCs with 120 days of overdue must adhere to the 90-day norm by March 31, 2025. The reference to "Base Layer NBFC" aligns with the context in [5], but the specific timeline for the glide path is derived from [1].</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12961_Undertaking-of-Financial-Services.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12949_Asset-Liability-Management.pdf p.10 | 12947_Resolution-of-Stressed-Assets.pdf p.15</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.17 | 12931_Miscellaneous.pdf p.14 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.10 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12949_Asset-Liability-Management.pdf p.10</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1021,7 +1017,7 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>9.199999999999999</v>
+        <v>13.4</v>
       </c>
       <c r="K11" t="inlineStr"/>
       <c r="L11" t="inlineStr"/>
@@ -1056,12 +1052,12 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>The provided context passages do not specify the minimum and maximum public-deposit tenors applicable to an eligible deposit-taking NBFC-ICC. The discussions in the passages focus on limits on deposit amounts [1], subscription norms for NCDs [2], credit ratings [3], applicability of concentration risk management [4], auditor reporting requirements [5], and definitions [6], but none address the duration (tenor) of public deposits for NBFC-ICC.</t>
+          <t>The context passages do not specify the minimum and maximum public-deposit tenors applicable to an eligible deposit-taking NBFC-ICC. The provided texts address prudential norms, credit ratings, NOF requirements, and applicability of regulations but do not mention deposit tenure limits for NBFC-ICC.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12931_Miscellaneous.pdf p.6 | 12958_Acceptance-of-Public-Deposits.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.2 | 13585_SUP-Auditors-Report.pdf p.4 | 12958_Acceptance-of-Public-Deposits.pdf p.4</t>
+          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.2 | 12958_Acceptance-of-Public-Deposits.pdf p.13 | 12958_Acceptance-of-Public-Deposits.pdf p.4 | 13585_SUP-Auditors-Report.pdf p.4 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -1075,7 +1071,7 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>11.5</v>
+        <v>9.5</v>
       </c>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
@@ -1110,26 +1106,26 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>The public-deposit ceiling for an eligible NBFC-ICC meeting the minimum NOF and prudential requirements is **one and one-half times its NOF**. This is specified in [1], which states that such an NBFC shall not accept or renew public deposits exceeding 1.5 times its NOF.</t>
+          <t>The public-deposit ceiling for an eligible NBFC-ICC meeting the minimum NOF and prudential requirements is **one and one-half times its NOF** [1]. This limit applies to accepting or renewing public deposits, with exceptions for matured deposits requiring explicit depositor consent [1].</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12939_Housing-Finance-Companies.pdf p.13 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.2</t>
+          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12939_Housing-Finance-Companies.pdf p.13 | 12944_Declaration-of-Dividends.pdf p.6 | 12953_Concentration-Risk-Management.pdf p.10 | 12958_Acceptance-of-Public-Deposits.pdf p.29</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>all key figures present (1.5times)</t>
+          <t>none of the expected figures appear (1.5times)</t>
         </is>
       </c>
       <c r="J13" t="n">
-        <v>8.4</v>
+        <v>7</v>
       </c>
       <c r="K13" t="inlineStr"/>
       <c r="L13" t="inlineStr"/>
@@ -1164,26 +1160,26 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>The minimum investment-grade credit rating prescribed for public-deposit acceptance is "minimum investment grade" as specified in the Reserve Bank of India (Non-Banking Financial Companies - Acceptance of Public Deposits) Directions, 2025. This requirement is explicitly mentioned in paragraphs 12 and 13 of the Directions [1], and further referenced in the auditor's report obligations [2]. No specific rating symbol (e.g., AAA, AA) is provided in the passages.</t>
+          <t>The context passages do not specify the exact minimum investment-grade credit rating required for public-deposit acceptance. They only state that NBFCs must obtain "minimum investment grade for fixed deposits" from an approved credit rating agency [1], but no particular rating level (e.g., AAA, BBB) is mentioned.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 13585_SUP-Auditors-Report.pdf p.4 | 12939_Housing-Finance-Companies.pdf p.51 | 12958_Acceptance-of-Public-Deposits.pdf p.14 | 12939_Housing-Finance-Companies.pdf p.38 | 12939_Housing-Finance-Companies.pdf p.38</t>
+          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 13585_SUP-Auditors-Report.pdf p.4 | 12958_Acceptance-of-Public-Deposits.pdf p.14 | 12939_Housing-Finance-Companies.pdf p.38 | 12939_Housing-Finance-Companies.pdf p.38 | 12958_Acceptance-of-Public-Deposits.pdf p.13</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CHECK</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>no numeric facts to compare - read the answer yourself</t>
+          <t>declined to answer an in-scope question - retrieval likely missed</t>
         </is>
       </c>
       <c r="J14" t="n">
-        <v>5.9</v>
+        <v>5.5</v>
       </c>
       <c r="K14" t="inlineStr"/>
       <c r="L14" t="inlineStr"/>
@@ -1218,12 +1214,12 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Recovery calls for overdue loans other than microfinance loans are prohibited outside the hours of 8:00 a.m. to 7:00 p.m. [1] (point 100). This restriction explicitly excludes microfinance loans under Reserve Bank of India directions [1]. Additionally, telemarketing contacts are generally restricted to 09:30 hours to 19:00 hours [4][6], but the specific prohibition for recovery calls applies to the 8:00 a.m.–7:00 p.m. window.</t>
+          <t>Recovery calls for overdue loans other than microfinance loans are prohibited outside the hours of 8:00 a.m. to 7:00 p.m. [1] (H.5, para 95) and [3] (H.4, para 91). Specifically, persistently calling before 8:00 a.m. or after 7:00 p.m. is deemed harsh and prohibited.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.28 | 12939_Housing-Finance-Companies.pdf p.70 | 12942_Responsible-Business-Conduct.pdf p.27 | 12939_Housing-Finance-Companies.pdf p.59 | 12942_Responsible-Business-Conduct.pdf p.9 | 12939_Housing-Finance-Companies.pdf p.58</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.28 | 12939_Housing-Finance-Companies.pdf p.70 | 12942_Responsible-Business-Conduct.pdf p.27 | 12942_Responsible-Business-Conduct.pdf p.9 | 12942_Responsible-Business-Conduct.pdf p.36 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -1237,7 +1233,7 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>12.8</v>
+        <v>13.4</v>
       </c>
       <c r="K15" t="inlineStr"/>
       <c r="L15" t="inlineStr"/>
@@ -1272,7 +1268,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>The minimum KFS validity period for retail and MSME term loans is **three working days** for loans with a tenor of **seven days or more**. For loans with a tenor of **less than seven days**, the validity period is **one working day** [1].</t>
+          <t>The minimum KFS validity period for retail and MSME term loans is **one working day** for loans with a tenor of less than seven days. For loans with a tenor of seven days or more, the validity period is at least three working days [1].</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1291,7 +1287,7 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>7.4</v>
+        <v>7.5</v>
       </c>
       <c r="K16" t="inlineStr"/>
       <c r="L16" t="inlineStr"/>
@@ -1326,12 +1322,12 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>A Middle Layer NBFC-ICC must appoint a Chief Risk Officer (CRO) if its asset size exceeds ₹5,000 crore. This is specified in [1], which states that NBFCs with asset size of more than ₹5,000 crore must appoint a CRO, regardless of their classification in the Middle Layer. The Middle Layer threshold (₹1,000 crore) is separate from the CRO requirement.</t>
+          <t>A Middle Layer NBFC-ICC must appoint a Chief Risk Officer (CRO) if its asset size exceeds ₹5,000 crore. This requirement is specified in [1], which mandates that NBFCs with asset sizes above ₹5,000 crore appoint a CRO, regardless of their classification in the Middle Layer. The Middle Layer classification itself is based on a separate threshold of ₹1,000 crore [5], but the CRO appointment criterion is distinct and tied to the ₹5,000 crore threshold.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 13588_SUP-Statutory-Audit.pdf p.7</t>
+          <t>12960_Governance.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -1345,7 +1341,7 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>7.3</v>
+        <v>9.6</v>
       </c>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
@@ -1380,12 +1376,12 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>A Middle Layer NBFC must submit its quarterly director-change statement and fit-and-proper certificate to the Regional Office of the RBI's Department of Supervision within **15 days of the close of the respective quarter** [1]. The statement for the quarter ending March 31 must also be **certified by the auditors** [1].</t>
+          <t>A Middle Layer NBFC must submit its quarterly director-change statement and fit-and-proper certificate to the Reserve Bank's Regional Office within **15 days of the close of the respective quarter**. The statement for the quarter ending **March 31** must be **certified by the auditors** [1].</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.9 | 12934_Peer-to-Peer-Lending-Platform.pdf p.17 | 12953_Concentration-Risk-Management.pdf p.2 | 12936_Account-Aggregator.pdf p.20 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12944_Declaration-of-Dividends.pdf p.6</t>
+          <t>12960_Governance.pdf p.9 | 12934_Peer-to-Peer-Lending-Platform.pdf p.17 | 12936_Account-Aggregator.pdf p.20 | 12953_Concentration-Risk-Management.pdf p.2 | 12960_Governance.pdf p.29 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -1435,12 +1431,12 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Under the November 28, 2025 version, routine credit-bureau reporting required submission of credit information on the 9th, 16th, 23rd, and last day of the month as reference dates [1]. For full-file submissions (containing all active and closed accounts as of the last day of the month), the deadline was the 5th day of the following month [1]. Incremental accounts for submissions on the 9th, 16th, and 23rd days must be reported within four calendar days of those dates [1].</t>
+          <t>The reference dates for routine credit-bureau reporting under the November 28, 2025 version are the 9th, 16th, 23rd, and last day of the month [1]. For the full file submission (containing all active accounts and ended relationships since the last reference date), the deadline is the 5th day of the next month [1]. Incremental accounts for the 9th, 16th, and 23rd must be submitted within four calendar days of those dates [1].</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>12955_Credit-Information-Reporting.pdf p.7 | 12955_Credit-Information-Reporting.pdf p.30 | 12955_Credit-Information-Reporting.pdf p.17 | 12954_Credit-Risk-Management.pdf p.27 | 12955_Credit-Information-Reporting.pdf p.14 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.40</t>
+          <t>12955_Credit-Information-Reporting.pdf p.7 | 12955_Credit-Information-Reporting.pdf p.30 | 12955_Credit-Information-Reporting.pdf p.17 | 12954_Credit-Risk-Management.pdf p.27 | 12955_Credit-Information-Reporting.pdf p.14 | 12955_Credit-Information-Reporting.pdf p.1</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -1454,7 +1450,7 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>6.7</v>
+        <v>12.2</v>
       </c>
       <c r="K19" t="inlineStr"/>
       <c r="L19" t="inlineStr"/>
@@ -1489,7 +1485,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>The minimum cooling-off period for a digital loan is one day, as stipulated in [1], which states that the NBFC must set the cooling-off period per their credit policy, subject to it not being less than one day.</t>
+          <t>The minimum cooling-off period for a digital loan is one day, as stipulated in [1], which states that the NBFC must determine the period "subject to the period so determined not being less than one day."</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1508,7 +1504,7 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>7.2</v>
+        <v>6.2</v>
       </c>
       <c r="K20" t="inlineStr"/>
       <c r="L20" t="inlineStr"/>
@@ -1543,26 +1539,26 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>The percentage cap applicable to default loss guarantee (DLG) cover on an eligible digital-lending portfolio is **five per cent** of the total amount disbursed from that loan portfolio at any given time. This is stipulated in the Cap on DLG provisions [2], which require NBFCs to ensure DLG cover does not exceed 5% of the disbursed amount. Additionally, this cap is referenced in provisions related to DLG arrangements under the Reserve Bank of India (Non-Banking Financial Companies - Credit Facilities) Directions, 2025 [5].</t>
+          <t>The percentage cap applicable to default loss guarantee (DLG) cover on an eligible digital-lending portfolio is **five per cent** of the total amount disbursed from that loan portfolio at any given time [3].</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.25 | 12957_Credit-Facilities.pdf p.24 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.22 | 12957_Credit-Facilities.pdf p.25 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.14 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.38</t>
+          <t>12959_Prudential-Norms-on-Capital-Adequacy.pdf p.25 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.22 | 12957_Credit-Facilities.pdf p.24 | 12957_Credit-Facilities.pdf p.25 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.14 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.38</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>REVIEW</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>all key figures present (5%)</t>
+          <t>none of the expected figures appear (5%)</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>8.1</v>
+        <v>5.8</v>
       </c>
       <c r="K21" t="inlineStr"/>
       <c r="L21" t="inlineStr"/>
@@ -1597,17 +1593,17 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>The Base, Middle, Upper, and Top Layers categorize Non-Banking Financial Companies (NBFCs) based on size, activity, and risk, with distinct regulatory and operational requirements:  
-- **Base Layer (NBFCs-BL)**: NBFCs with smaller size and lower risk, such as NBFC-P2P, NBFC-AA, NOFHC, and Type I NBFCs [3]. Materiality thresholds for loans are ₹1 crore [2]. Regulatory compliance includes Chapter III only [5].  
-- **Middle Layer (NBFCs-ML)**: NBFCs with moderate size/risk, including HFCs, IFCs, SPD, and IDF-NBFCs [3]. Materiality thresholds are ₹5 crore [2]. Regulatory compliance includes Chapters II, III, and IV [5]. Governance requires EWS frameworks [6].  
-- **Upper Layer (NBFCs-UL)**: Larger, higher-risk NBFCs (e.g., NBFC-D, CIC, NBFC-IFC) with materiality thresholds of ₹10 crore [2]. Regulatory compliance includes Chapters II, III, IV, and V [5]. Governance mandates EWS frameworks and stricter oversight [6].  
-- **Top Layer (NBFCs-TL)**: Ideally empty, but if populated, would represent the highest-risk NBFCs with the strictest regulations [1].  
-Layer classification depends on asset size, activity, and supervisory assessments [4].</t>
+          <t>The Base, Middle, Upper, and Top Layers categorize NBFCs based on size, activity, and risk, with distinct regulatory requirements:  
+- **Base Layer (NBFCs-BL)**: Includes small NBFCs (e.g., NBFC-P2P, NBFC-AA, NOFHC, and Type I NBFCs) and certain existing NBFC-ND-SI with asset sizes ₹500 crore–₹1,000 crore. Materiality threshold for loans: ₹1 crore [3].  
+- **Middle Layer (NBFCs-ML)**: Applies to NBFC-D, CIC, NBFC-IFC, HFC, SPD, IDF-NBFC, and others (e.g., NBFC-Investment and Credit Companies). Materiality threshold: ₹5 crore [3]. Minimum Tier 1 capital: 10% of RWAs; CRAR: 15% [5].  
+- **Upper Layer (NBFCs-UL)**: Applies to larger NBFCs (e.g., NBFC-ND-SI above ₹1,000 crore). Materiality threshold: ₹10 crore [3]. Minimum CET1 capital: 9% of RWAs [5].  
+- **Top Layer (NBFCs-TL)**: Ideally empty, but if populated, subject to higher capital charges [1].  
+These layers determine regulatory capital, lending thresholds, and categorization for specific NBFC types [1][2][4][5].</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12954_Credit-Risk-Management.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12960_Governance.pdf p.3 | 13590_SUP-Fraud-Risk-Management.pdf p.10</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12954_Credit-Risk-Management.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12937_Core-Investment-Companies.pdf p.6</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -1621,7 +1617,7 @@
         </is>
       </c>
       <c r="J22" t="n">
-        <v>9.300000000000001</v>
+        <v>9.6</v>
       </c>
       <c r="K22" t="inlineStr"/>
       <c r="L22" t="inlineStr"/>
@@ -1656,12 +1652,12 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Not taking customer deposits does not necessarily mean an NBFC does not use public funds. According to [1], 'public funds' include funds raised through public deposits, inter-corporate deposits, bank finance, and other sources like Commercial Papers or debentures [18]. Thus, even if an NBFC avoids customer deposits (public deposits), it could still use other forms of public funds. The distinction hinges on whether the NBFC accepts any of these broader categories of public funds.</t>
+          <t>Not taking customer deposits does not automatically mean a company does not use public funds. According to [1](#1), 'public funds' include funds raised through public deposits, inter-corporate deposits, bank finance, and other external sources like Commercial Papers or debentures [1](#1). Even if a company does not accept customer deposits, it could still use public funds via these alternative channels. Additionally, [5](#5) defines 'public deposit' as a specific type of deposit excluded from certain entities, but public funds encompass broader sources. Thus, avoiding customer deposits does not equate to avoiding all public funds.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.27 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.18 | 13585_SUP-Auditors-Report.pdf p.6 | 12958_Acceptance-of-Public-Deposits.pdf p.2 | 12958_Acceptance-of-Public-Deposits.pdf p.6</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.27 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.18 | 13585_SUP-Auditors-Report.pdf p.6 | 12958_Acceptance-of-Public-Deposits.pdf p.6 | 12937_Core-Investment-Companies.pdf p.10</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -1675,7 +1671,7 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>6.5</v>
+        <v>6.3</v>
       </c>
       <c r="K23" t="inlineStr"/>
       <c r="L23" t="inlineStr"/>
@@ -1710,12 +1706,12 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>No, once a customer's KYC documents are checked, monitoring of their transactions cannot be stopped. The NBFC must ensure periodic updation of KYC data, with intervals based on risk categories: high-risk customers require updates every 2 years, medium-risk every 8 years, and low-risk every 10 years [6]. Additionally, accounts opened via OTP-based e-KYC must undergo CDD within 1 year; otherwise, operations are suspended [4]. Failure to comply with periodic KYC updates may result in temporary cessation of account operations [5]. Thus, ongoing monitoring and verification are mandated.</t>
+          <t>No, the passages indicate that ongoing monitoring is required even after initial KYC checks. For example, accounts must be monitored for suspicion of ML/TF activities [1](28(viii)), transaction limits apply [5](25(3)-(4)), and periodic KYC updation is mandated based on risk categories [6](42(1)). Additionally, failure to comply with KYC requirements triggers account suspension [1](28(vi)).</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>12943_Know-Your-Customer.pdf p.34 | 12943_Know-Your-Customer.pdf p.56 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.28 | 12943_Know-Your-Customer.pdf p.44 | 12943_Know-Your-Customer.pdf p.41</t>
+          <t>12943_Know-Your-Customer.pdf p.34 | 12943_Know-Your-Customer.pdf p.6 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.57 | 12943_Know-Your-Customer.pdf p.28 | 12943_Know-Your-Customer.pdf p.41</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -1729,7 +1725,7 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>8.699999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="K24" t="inlineStr"/>
       <c r="L24" t="inlineStr"/>
@@ -1769,7 +1765,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>12943_Know-Your-Customer.pdf p.19 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.7 | 12943_Know-Your-Customer.pdf p.45 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.7 | 12943_Know-Your-Customer.pdf p.32</t>
+          <t>12943_Know-Your-Customer.pdf p.19 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.7 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.45 | 12943_Know-Your-Customer.pdf p.30 | 12943_Know-Your-Customer.pdf p.28</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1783,7 +1779,7 @@
         </is>
       </c>
       <c r="J25" t="n">
-        <v>5.7</v>
+        <v>5.2</v>
       </c>
       <c r="K25" t="inlineStr"/>
       <c r="L25" t="inlineStr"/>
@@ -1818,7 +1814,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>No, sending every borrower an English-only loan letter is not sufficient. The passages mandate that communications with borrowers must be in the vernacular language or a language as understood by the borrower [1], [2], [3]. For illiterate borrowers, terms and conditions must be explained in the presence of a witness, and all critical documents, including loan agreements and Key Fact Statements (KFS), must be in the language of the region or the language chosen by the borrower [3], [4]. English-only communication would violate these requirements unless the borrower explicitly understands English.</t>
+          <t>No, sending every borrower an English-only loan letter is not sufficient. The passages mandate that communications must be in the vernacular language or a language as understood by the borrower [1], [2], [3]. For illiterate borrowers, terms and conditions must be explained in the presence of a witness, not necessarily in English [3]. English-only communication would fail to meet these requirements for borrowers who do not understand English.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1837,7 +1833,7 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>5.9</v>
+        <v>5.1</v>
       </c>
       <c r="K26" t="inlineStr"/>
       <c r="L26" t="inlineStr"/>
@@ -1872,7 +1868,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Yes, borrowers must receive copies of all enclosures quoted in the loan agreement. According to the regulations, an NBFC shall "furnish a copy of the loan agreement along with a copy each of all enclosures quoted in the loan agreement to all the borrowers at the time of sanction/disbursement of loans" [1]. This requirement is reiterated in [2] and [3], emphasizing that such copies are necessary to ensure transparency and prevent disputes over terms and conditions.</t>
+          <t>Yes, borrowers must receive copies of all enclosures quoted in the loan agreement. According to [1], NBFCs are required to furnish a copy of the loan agreement **along with a copy each of all enclosures quoted in the loan agreement** to borrowers at the time of sanction/disbursement. Similarly, [2] mandates that a copy of the terms and conditions (including enclosures) must be made available to the borrower. [3] and [4] further reinforce this requirement, emphasizing that all applicable charges, collateral details, and procedural terms must be included in the loan agreement and provided to borrowers. Thus, copies of all attachments are explicitly mandated.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1891,7 +1887,7 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>5.8</v>
+        <v>7.1</v>
       </c>
       <c r="K27" t="inlineStr"/>
       <c r="L27" t="inlineStr"/>
@@ -1926,12 +1922,12 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>The Board of an NBFC or HFC should decide how to set lending rates, considering factors such as cost of funds, margin, and risk premium [1], [3], [5]. They must also account for the nature of services provided, quantum of loans, and other objective parameters [5]. Additionally, they must ensure transparency by disclosing these factors to borrowers and aligning with regulatory norms and the Fair Practices Code [1], [4].</t>
+          <t>The Board of an NBFC or HFC should decide lending rates, considering factors such as cost of funds, margin, and risk premium [1], [3], [5]. They must also account for the borrower's risk profile and ensure transparency in communication [1], [5]. For microfinance loans, additional considerations include setting ceilings on interest rates and charges, and ensuring non-usurious pricing [3]. The Board's policy must delineate these components and their quantum based on objective parameters [3].</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.10 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.36 | 12939_Housing-Finance-Companies.pdf p.12 | 12939_Housing-Finance-Companies.pdf p.56 | 12957_Credit-Facilities.pdf p.37 | 12942_Responsible-Business-Conduct.pdf p.16</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.10 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.36 | 12957_Credit-Facilities.pdf p.37 | 12939_Housing-Finance-Companies.pdf p.56 | 12939_Housing-Finance-Companies.pdf p.12 | 12942_Responsible-Business-Conduct.pdf p.16</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -1945,7 +1941,7 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>5.5</v>
+        <v>6.3</v>
       </c>
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
@@ -1980,12 +1976,12 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Yes, the Board of an NBFC must disclose the rationale for charging different interest rates to different categories of borrowers. The rate of interest and the approach for gradations of risk must be explicitly communicated in the sanction letter and application form, explaining the basis for differential rates [1].</t>
+          <t>Yes, the Board of an NBFC must disclose the rationale for charging different interest rates to different categories of borrowers. This includes explaining the factors such as cost of funds, margin, and risk premium used in determining the rates, which must be communicated explicitly in the sanction letter and application form [1].</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.10 | 12942_Responsible-Business-Conduct.pdf p.16 | 12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.4 | 12951_Securitisation-Transactions.pdf p.23 | 12947_Resolution-of-Stressed-Assets.pdf p.54</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.10 | 12942_Responsible-Business-Conduct.pdf p.16 | 12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.4 | 12951_Securitisation-Transactions.pdf p.23 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.13</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -2034,12 +2030,12 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>No, it is not solely the agency's problem. The HFC/NBFC retains responsibility for ensuring recovery agents adhere to legal and ethical standards. For instance, HFCs must ensure contracts with recovery agents do not incentivize uncivilized behavior [1], and NBFCs are liable for their agents' actions, including harassment or intimidation [2]. Additionally, HFCs must address borrower grievances before involving recovery agents [5], and NBFCs must ensure agents comply with fair practices codes [4]. Thus, the HFC/NBFC shares accountability for the agency's conduct.</t>
+          <t>No, it is not solely the agency's problem. The HFC/NBFC/card issuer has responsibilities to ensure recovery agents adhere to guidelines, including preventing mistreatment. For example, HFCs must ensure contracts with recovery agents do not induce unlawful behavior [1], and NBFCs must vet agents via due diligence and police verification [2]. Card issuers are liable for their agents' actions, including harassment [3]. Additionally, lenders must monitor agents, address grievances, and ensure compliance with fair practices codes [4][5]. Thus, the lender shares responsibility for ensuring proper conduct.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>12939_Housing-Finance-Companies.pdf p.70 | 12942_Responsible-Business-Conduct.pdf p.28 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.19 | 12942_Responsible-Business-Conduct.pdf p.27 | 12939_Housing-Finance-Companies.pdf p.72 | 12942_Responsible-Business-Conduct.pdf p.9</t>
+          <t>12939_Housing-Finance-Companies.pdf p.70 | 12942_Responsible-Business-Conduct.pdf p.28 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.19 | 12942_Responsible-Business-Conduct.pdf p.27 | 12939_Housing-Finance-Companies.pdf p.72 | 12942_Responsible-Business-Conduct.pdf p.36</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -2053,7 +2049,7 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>7.1</v>
+        <v>8.5</v>
       </c>
       <c r="K30" t="inlineStr"/>
       <c r="L30" t="inlineStr"/>
@@ -2088,12 +2084,12 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>No, an NBFC does not require prior approval from RBI to outsource financial services. The RBI does not mandate approval for such contracts, but the arrangements are subject to on-site/offsite monitoring and inspection by RBI [1].</t>
+          <t>No, RBI does not require prior approval for every financial-services outsourcing contract. An NBFC may outsource financial services without prior RBI approval, though such arrangements are subject to RBI monitoring, inspection, and scrutiny [1]. The NBFC must ensure compliance with regulatory requirements through written agreements, audits, and risk management practices, but explicit prior approval from RBI is not mandated for signing contracts.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>12941_Managing-Risks-in-Outsourcing.pdf p.13 | 12941_Managing-Risks-in-Outsourcing.pdf p.18 | 12941_Managing-Risks-in-Outsourcing.pdf p.32 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12941_Managing-Risks-in-Outsourcing.pdf p.21 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.25</t>
+          <t>12941_Managing-Risks-in-Outsourcing.pdf p.13 | 12941_Managing-Risks-in-Outsourcing.pdf p.18 | 12941_Managing-Risks-in-Outsourcing.pdf p.32 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.25 | 12941_Managing-Risks-in-Outsourcing.pdf p.21</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -2107,7 +2103,7 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>4.7</v>
+        <v>5.9</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -2147,7 +2143,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>12955_Credit-Information-Reporting.pdf p.7 | 12955_Credit-Information-Reporting.pdf p.8 | 12955_Credit-Information-Reporting.pdf p.13 | 12955_Credit-Information-Reporting.pdf p.10 | 12955_Credit-Information-Reporting.pdf p.28 | 12955_Credit-Information-Reporting.pdf p.20</t>
+          <t>12955_Credit-Information-Reporting.pdf p.7 | 12955_Credit-Information-Reporting.pdf p.8 | 12955_Credit-Information-Reporting.pdf p.13 | 12955_Credit-Information-Reporting.pdf p.10 | 12955_Credit-Information-Reporting.pdf p.20 | 12955_Credit-Information-Reporting.pdf p.28</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -2161,7 +2157,7 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -2196,12 +2192,12 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>No, the prohibition in [1] explicitly states that NBFCs cannot accept public deposits repayable on demand. Additionally, [4] allows premature repayment only after three months from the deposit date, which is not equivalent to on-demand access. Thus, the product cannot function like a savings account with immediate repayment flexibility.</t>
+          <t>No, the NBFC cannot accept public deposits repayable on demand. According to [1], "No NBFC shall accept any public deposit which is repayable on demand." While premature repayment may be allowed under specific conditions (e.g., after three months) [4], this does not equate to on-demand accessibility. The prohibition on demand deposits explicitly restricts customers from demanding repayment at any time.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12958_Acceptance-of-Public-Deposits.pdf p.37 | 12958_Acceptance-of-Public-Deposits.pdf p.17 | 12958_Acceptance-of-Public-Deposits.pdf p.20 | 12958_Acceptance-of-Public-Deposits.pdf p.18 | 12949_Asset-Liability-Management.pdf p.28</t>
+          <t>12958_Acceptance-of-Public-Deposits.pdf p.13 | 12958_Acceptance-of-Public-Deposits.pdf p.37 | 12958_Acceptance-of-Public-Deposits.pdf p.17 | 12958_Acceptance-of-Public-Deposits.pdf p.20 | 12958_Acceptance-of-Public-Deposits.pdf p.18 | 12958_Acceptance-of-Public-Deposits.pdf p.39</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -2215,7 +2211,7 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>5.8</v>
+        <v>6.3</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
@@ -2250,7 +2246,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>For an ordinary loan that has become a Non-Performing Asset (NPA), **unpaid interest cannot be booked as income**. Income recognition for NPAs is restricted to when it is *actually realised*. Any income recognised before the asset became non-performing and remaining unrealised must be reversed [2]§38. This applies regardless of the loan type, unless specific exceptions (e.g., moratorium periods) apply [2]§40.</t>
+          <t>For an ordinary loan that has become a Non-Performing Asset (NPA), **unpaid interest cannot be booked as income**. Income on NPAs, including interest, is recognized **only when actually realized**. Any income recognized before the asset became non-performing and remaining unrealized must be **reversed** [2]. This applies to all NPAs, including loans, as per the income recognition rules.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2269,7 +2265,7 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
       <c r="K34" t="inlineStr"/>
       <c r="L34" t="inlineStr"/>
@@ -2304,26 +2300,26 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>The provided context passages do not mention whether a Middle Layer NBFC requires a designated compliance head. The discussions focus on regulatory layers, fraud risk management committees, and compliance with specific chapters of governance directions, but none explicitly address the need for a compliance head.</t>
+          <t>Yes, a Middle Layer NBFC requires a designated compliance head. Specifically, it must appoint a Chief Compliance Officer (CCO), as mandated by Board-approved policies for Middle Layer and Upper Layer NBFCs [1]. The CCO must be a senior executive with a position not below two levels from the CEO (or one level further relaxed for Middle Layer NBFCs) [4]. Additionally, the NBFC must ensure the CCO has direct reporting lines to the MD/CEO or Board/Audit Committee (ACB) [4]. This role is explicitly required under the regulatory framework for Middle Layer NBFCs.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>12953_Concentration-Risk-Management.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.10 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 12960_Governance.pdf p.3 | 13590_SUP-Fraud-Risk-Management.pdf p.7 | 13590_SUP-Fraud-Risk-Management.pdf p.10</t>
+          <t>12960_Governance.pdf p.7 | 12960_Governance.pdf p.29 | 13590_SUP-Fraud-Risk-Management.pdf p.7 | 13593_SUP-Compliance-Function.pdf p.10 | 13593_SUP-Compliance-Function.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>CHECK</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>declined to answer an in-scope question - retrieval likely missed</t>
+          <t>no numeric facts to compare - read the answer yourself</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>8.1</v>
+        <v>7.6</v>
       </c>
       <c r="K35" t="inlineStr"/>
       <c r="L35" t="inlineStr"/>
@@ -2358,7 +2354,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>The vendor's promise alone is not sufficient. The outsourcing agreement must include specific contingency plans to ensure testing requirements [1](x), business continuity measures [2](f), and provisions for risk mitigation strategies [4](15). Additionally, the agreement must grant the NBFC or HFC rights to audit the service provider [1](ii), access IT infrastructure [1](xii), and enforce termination clauses [2](d). These requirements are explicitly outlined in the regulatory frameworks, indicating that contractual clauses and documented safeguards, not mere promises, are necessary.</t>
+          <t>The vendor's promise alone is not sufficient. The outsourcing agreement must include specific contingency plans to ensure business continuity, as explicitly required in the context passages. For example, [1](x) mandates contingency plan(s) to ensure testing requirements, and [2](f) states that contingency plans must be included to ensure business continuity. Additionally, the agreement must contain clauses addressing risk management, audit rights, and liability for subcontractors [1](xiii), [1](x), and [2](h). These requirements go beyond a mere promise, necessitating contractual safeguards and actionable measures.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2377,7 +2373,7 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>7.5</v>
+        <v>6.8</v>
       </c>
       <c r="K36" t="inlineStr"/>
       <c r="L36" t="inlineStr"/>
@@ -2412,12 +2408,13 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>No, the two NBFC-ICCs cannot both remain in the Base Layer. According to [1], if the consolidated asset size of NBFCs in a group reaches ₹1000 crore or more, all NBFCs in the group (including NBFC-ICC) are classified as Middle Layer. In this case, the consolidated assets of ₹600 crore + ₹500 crore = ₹1100 crore exceed the ₹1000 crore threshold, triggering Middle Layer classification for both NBFC-ICCs. [3] further clarifies that NBFC-ICC is by default in the Base Layer unless consolidation pushes them to Middle Layer. Thus, they must be classified in the Middle Layer.</t>
+          <t>The consolidated assets of the two NBFC-ICCs (₹600 crore + ₹500 crore = ₹1100 crore) exceed the ₹1000 crore threshold for Middle Layer classification [1]. Under paragraph 18 of [1], NBFC-ICC in a group with consolidated assets ≥ ₹1000 crore must be classified in the Middle Layer. Thus, **both NBFC-ICCs cannot remain in the Base Layer**; they would be classified in the Middle Layer. 
+Additionally, NBFC-ICC is by default in the Base Layer on a standalone basis [3], but group consolidation overrides this for classification purposes.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.3 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.2 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13592_SUP-Cybersecurity-Technology-Risk-Resilience.pdf p.3 | 12936_Account-Aggregator.pdf p.3 | 12953_Concentration-Risk-Management.pdf p.2</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -2431,7 +2428,7 @@
         </is>
       </c>
       <c r="J37" t="n">
-        <v>10.3</v>
+        <v>9.1</v>
       </c>
       <c r="K37" t="inlineStr"/>
       <c r="L37" t="inlineStr"/>
@@ -2466,12 +2463,12 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>No, you cannot immediately stop Middle Layer reporting. According to [1], if an NBFC's asset size falls below ₹1,000 crore due to temporary fluctuations, it must continue complying with Middle Layer reporting requirements and extant directions until the submission of its next audited balance sheet to the Reserve Bank and a specific dispensation is granted. Temporary declines in asset size do not exempt NBFCs from ongoing obligations until formal reassessment by the RBI.</t>
+          <t>No, you cannot immediately stop Middle Layer reporting. According to [1], if an NBFC's asset size falls below ₹1,000 crore due to temporary fluctuations, it must continue complying with NBFC-ML reporting requirements and regulations until the submission of its next audited balance sheet to the Reserve Bank or a specific dispensation is granted. Temporary declines in asset size do not exempt NBFCs from ongoing compliance with Middle Layer obligations.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.11 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13587_SUP-Supervisory-Returns.pdf p.8</t>
+          <t>12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13 | 13587_SUP-Supervisory-Returns.pdf p.8 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.21 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.13</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -2485,7 +2482,7 @@
         </is>
       </c>
       <c r="J38" t="n">
-        <v>6.6</v>
+        <v>5.6</v>
       </c>
       <c r="K38" t="inlineStr"/>
       <c r="L38" t="inlineStr"/>
@@ -2520,12 +2517,12 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>The NBFC-ICC as a Middle Layer NBFC must maintain a minimum Tier 1 capital of 10% of aggregate RWAs [3]. With only 9% Tier 1 capital, it fails to meet this requirement. While its CRAR of 17% exceeds the 15% minimum for Middle Layer NBFCs [3], Tier 1 capital alone must meet the 10% threshold. Thus, the NBFC is not capital-compliant.</t>
+          <t>The NBFC-ICC as a Middle Layer NBFC must maintain a minimum Tier 1 capital of 10% of aggregate RWAs [5]. With only 9% Tier 1 capital, it is **not compliant**. While the CRAR of 17% exceeds the 15% minimum for Middle Layer NBFCs [5], Tier 1 capital requirements are separate and mandatory. The Tier 2 capital cannot exceed 100% of Tier 1 capital [5], but the shortfall in Tier 1 capital (9% vs. required 10%) renders the entity non-compliant regardless of CRAR.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>12953_Concentration-Risk-Management.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.2 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12944_Declaration-of-Dividends.pdf p.6 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 13586_SUP-Miscellaneous.pdf p.8</t>
+          <t>12953_Concentration-Risk-Management.pdf p.10 | 13586_SUP-Miscellaneous.pdf p.8 | 12944_Declaration-of-Dividends.pdf p.6 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.13 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.7 | 12953_Concentration-Risk-Management.pdf p.2</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -2539,7 +2536,7 @@
         </is>
       </c>
       <c r="J39" t="n">
-        <v>9.199999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="K39" t="inlineStr"/>
       <c r="L39" t="inlineStr"/>
@@ -2574,12 +2571,12 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>If the NBFC forms a suspicion of money laundering or terrorist financing and reasonably believes that performing the CDD process will tip off the customer, it shall not pursue the CDD process and instead file an STR with FIU-IND [1]. Thus, in such circumstances, further KYC questioning should not continue.</t>
+          <t>If the NBFC forms a suspicion of money laundering or terrorist financing and reasonably believes that performing the CDD process would tip off the customer, it shall not pursue the CDD process and instead file an STR with FIU-IND [1]. Thus, in such circumstances, further KYC questioning should be avoided to prevent alerting the customer.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>12943_Know-Your-Customer.pdf p.19 | 12931_Miscellaneous.pdf p.9 | 12943_Know-Your-Customer.pdf p.15 | 12943_Know-Your-Customer.pdf p.56 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.16</t>
+          <t>12943_Know-Your-Customer.pdf p.19 | 12931_Miscellaneous.pdf p.9 | 12943_Know-Your-Customer.pdf p.15 | 12943_Know-Your-Customer.pdf p.42 | 12943_Know-Your-Customer.pdf p.57 | 12943_Know-Your-Customer.pdf p.16</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
@@ -2593,7 +2590,7 @@
         </is>
       </c>
       <c r="J40" t="n">
-        <v>6.1</v>
+        <v>5.9</v>
       </c>
       <c r="K40" t="inlineStr"/>
       <c r="L40" t="inlineStr"/>
@@ -2628,12 +2625,12 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>No, the loan cannot become standard. According to paragraph 25 of [1], loan accounts classified as NPA may be upgraded to standard only upon repayment of **entire arrears of interest and principal pertaining to all** credit facilities. Since the borrower has cleared arrears for only one of the two loans, the entire account (both loans) remains classified as NPA. Additionally, paragraph 24 of [1] specifies that an NPA can be upgraded to standard only if **entire arrears** (interest and principal) are paid, which is not satisfied here.</t>
+          <t>No. According to paragraph 25 of [1], loan accounts classified as NPAs may be upgraded to standard only upon repayment of **entire arrears of interest and principal pertaining to all** credit facilities. Since the borrower has two loans (facilities) classified as NPA, clearing arrears on **only one** does not satisfy the requirement for upgradation. The entire arrears across **all** facilities must be repaid for the account to be reclassified as standard [1].</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12947_Resolution-of-Stressed-Assets.pdf p.52 | 12957_Credit-Facilities.pdf p.29 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12</t>
+          <t>12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.8 | 12957_Credit-Facilities.pdf p.29 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.24 | 12947_Resolution-of-Stressed-Assets.pdf p.52 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.20 | 12947_Resolution-of-Stressed-Assets.pdf p.35</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
@@ -2647,7 +2644,7 @@
         </is>
       </c>
       <c r="J41" t="n">
-        <v>7.9</v>
+        <v>8</v>
       </c>
       <c r="K41" t="inlineStr"/>
       <c r="L41" t="inlineStr"/>
@@ -2682,12 +2679,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>The digital-lending partner's request to receive disbursements in its own pool account and then transfer them to borrowers is **not permitted**. 
-Under the regulations, NBFC-P2P platforms are prohibited from holding funds received from lenders on their own balance sheet, including through pool accounts. Specifically:  
-- Funds from lenders must be transferred to the **Lenders' Escrow Account** and disbursed directly to the borrower's bank account **after compliance with paragraph 34** [1].  
-- The NBFC-P2P **cannot hold funds** for servicing loans or use pool accounts for this purpose, as this would violate the requirement that "funds received from lenders... shall not be held on its own balance sheet" [3].  
-- All fund transfers must occur **through and from bank accounts**, with **cash transactions strictly prohibited** [1].  
-Thus, the proposed mechanism involving a pool account would breach these prudential norms.</t>
+          <t>The digital-lending partner (LSP) cannot receive disbursements into its own pool account. According to passage [2], loan servicing, repayment, etc., must be executed "directly in the NBFC's account without any pass-through account or pool account of any third party" [2]. Additionally, passage [3] prohibits NBFC-P2P entities from holding funds received from lenders or borrowers in their own balance sheets [3]. While the LSP may facilitate disbursements, the mechanism must avoid third-party pool accounts, as such arrangements are explicitly disallowed under the prudential norms. Thus, the proposed method is not permitted.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2706,7 +2698,7 @@
         </is>
       </c>
       <c r="J42" t="n">
-        <v>8.800000000000001</v>
+        <v>9</v>
       </c>
       <c r="K42" t="inlineStr"/>
       <c r="L42" t="inlineStr"/>
@@ -2741,12 +2733,12 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Consent alone is not sufficient. The NBFC must ensure that data collection is need-based, with prior and explicit consent, and that the consent artefact includes standardized details such as the purpose of data collection, recipients, and revocation rights [1][3]. Access to mobile resources like contact lists is explicitly prohibited unless for onboarding/KYC purposes [1]. Since credit scoring is not explicitly listed as a permitted purpose for contact list access, even with consent, the practice may violate regulations.</t>
+          <t>Consent alone is not sufficient. According to [2], NBFCs must ensure data collection by their DLA and LSP is need-based and with prior, explicit consent. However, access to mobile phone resources like contact lists is explicitly prohibited unless for onboarding/KYC purposes, with one-time access only. Since the app's purpose (credit scoring) is not part of onboarding, accessing the contact list would violate these guidelines. Consent is required but not sufficient on its own for such access.</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>12957_Credit-Facilities.pdf p.19 | 12955_Credit-Information-Reporting.pdf p.8 | 12936_Account-Aggregator.pdf p.13 | 12934_Peer-to-Peer-Lending-Platform.pdf p.12 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.18 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.7</t>
+          <t>12955_Credit-Information-Reporting.pdf p.8 | 12957_Credit-Facilities.pdf p.19 | 12936_Account-Aggregator.pdf p.13 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.18 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.7 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.6</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
@@ -2760,7 +2752,7 @@
         </is>
       </c>
       <c r="J43" t="n">
-        <v>9.800000000000001</v>
+        <v>9.1</v>
       </c>
       <c r="K43" t="inlineStr"/>
       <c r="L43" t="inlineStr"/>
@@ -2795,12 +2787,12 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>No, an NBFC cannot automatically increase credit limits for customers who repay on time. According to [2](2), an NBFC shall ensure there is no automatic increase in credit limit unless an explicit request is received, evaluated, and kept on record from the borrower. Automatic adjustments without such a request are prohibited.</t>
+          <t>No, an NBFC cannot automatically increase credit limits for customers who repay on time. According to [1] §8(2), an NBFC must ensure there is no automatic increase in credit limits unless an explicit request is received, evaluated, and kept on record from the borrower. The passage explicitly prohibits automatic adjustments without borrower-initiated action.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>13591_SUP-Digital-Payment-Security-Controls.pdf p.6 | 12957_Credit-Facilities.pdf p.15 | 12942_Responsible-Business-Conduct.pdf p.16 | 12942_Responsible-Business-Conduct.pdf p.18 | 12943_Know-Your-Customer.pdf p.40 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.7</t>
+          <t>12957_Credit-Facilities.pdf p.15 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.6 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.14 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.18 | 13591_SUP-Digital-Payment-Security-Controls.pdf p.27 | 12957_Credit-Facilities.pdf p.8</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
@@ -2814,7 +2806,7 @@
         </is>
       </c>
       <c r="J44" t="n">
-        <v>5.7</v>
+        <v>6.3</v>
       </c>
       <c r="K44" t="inlineStr"/>
       <c r="L44" t="inlineStr"/>
@@ -2849,12 +2841,12 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>The decision to sanction retail loans is explicitly listed as a core management function that **shall not be outsourced** [1]. This prohibition applies regardless of the NBFC's layer (including Middle Layer). While Middle Layer NBFCs are subject to specific outsourcing provisions [2], the sanctioning of loans (including retail loans) remains a non-outsourcable function. Thus, outsourcing this decision to an unrelated fintech vendor is not permitted.</t>
+          <t>No, you cannot outsource the final decision to sanction retail loans. According to [1], NBFCs are prohibited from outsourcing "decision-making functions such as determining compliance with KYC norms for opening deposit accounts, giving sanction for loans (including retail loans)" as part of core management functions. This restriction applies regardless of the NBFC's layer (Middle Layer or otherwise). The prohibition explicitly includes retail loan sanctioning decisions, even when engaging unrelated vendors.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>12941_Managing-Risks-in-Outsourcing.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12941_Managing-Risks-in-Outsourcing.pdf p.24 | 12954_Credit-Risk-Management.pdf p.13 | 12957_Credit-Facilities.pdf p.14 | 12941_Managing-Risks-in-Outsourcing.pdf p.13</t>
+          <t>12941_Managing-Risks-in-Outsourcing.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4 | 12941_Managing-Risks-in-Outsourcing.pdf p.24 | 12954_Credit-Risk-Management.pdf p.13 | 12957_Credit-Facilities.pdf p.14 | 12941_Managing-Risks-in-Outsourcing.pdf p.37</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
@@ -2868,7 +2860,7 @@
         </is>
       </c>
       <c r="J45" t="n">
-        <v>7.6</v>
+        <v>6.9</v>
       </c>
       <c r="K45" t="inlineStr"/>
       <c r="L45" t="inlineStr"/>
@@ -2903,7 +2895,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>No, you cannot skip a formal outsourcing agreement. The context explicitly requires that even when outsourcing to a group entity (related party), the NBFC must ensure the arrangement is documented in a legally binding written agreement with detailed terms, including service scope, confidentiality, audit rights, and risk management provisions [1], [4], [5]. Additionally, the agreement must allow the NBFC to maintain control, ensure compliance with regulatory oversight (e.g., RBI inspections), and include clauses for termination and data protection [1], [4], [5]. Risk management practices for group entities are identical to those for non-related parties [1].</t>
+          <t>No, the passages explicitly require formal outsourcing agreements even when outsourcing to group entities. For example, [1] states that NBFCs must have Service Level Agreements (SLAs) with group entities, and [5] mandates that outsourcing arrangements be governed by written agreements vetted by legal counsel. Additionally, [4] and [6] outline specific contractual clauses (e.g., data confidentiality, audit rights, termination terms) that must be included regardless of the relationship between the entities. The shared parent company does not exempt the NBFC from these requirements.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2922,7 +2914,7 @@
         </is>
       </c>
       <c r="J46" t="n">
-        <v>9.6</v>
+        <v>7.9</v>
       </c>
       <c r="K46" t="inlineStr"/>
       <c r="L46" t="inlineStr"/>
@@ -2957,12 +2949,12 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>No, it is not allowed. Key Managerial Personnel (KMP) of an NBFC in the Middle Layer (NBFC-ML) cannot hold directorships in other NBFC-ML or NBFC-UL entities unless the position is in a subsidiary. The CFO, as KMP, cannot assume directorship in another Middle Layer NBFC that is not a subsidiary [1].</t>
+          <t>No, it is not allowed. Key Managerial Personnel (KMP) of an NBFC shall not hold any office, including directorships, in another NBFC-ML (Middle Layer) or NBFC-UL (Upper Layer) entity, except for directorships in NBFC-BL (Base Layer) [1]. Since the other NBFC is also in the Middle Layer, the CFO cannot assume directorship there.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>12960_Governance.pdf p.12 | 12960_Governance.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12944_Declaration-of-Dividends.pdf p.6 | 12946_Wilful-Defaulters-and-Large-Defaulters.pdf p.3 | 12961_Undertaking-of-Financial-Services.pdf p.2</t>
+          <t>12960_Governance.pdf p.12 | 12953_Concentration-Risk-Management.pdf p.2 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12960_Governance.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.12 | 12941_Managing-Risks-in-Outsourcing.pdf p.4</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -2976,7 +2968,7 @@
         </is>
       </c>
       <c r="J47" t="n">
-        <v>7.4</v>
+        <v>6.3</v>
       </c>
       <c r="K47" t="inlineStr"/>
       <c r="L47" t="inlineStr"/>
@@ -3011,7 +3003,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>No, the NBFC cannot renew existing public deposits if its credit rating has been downgraded below the minimum investment grade. According to [1], in such cases, the NBFC must immediately stop accepting fresh public deposits and renewing existing ones. Additionally, [2] states that if public deposits exceed one and one-half times the NOF, the NBFC cannot renew or accept fresh deposits until the limit is restored. Thus, during the downgraded period, renewals are prohibited.</t>
+          <t>If an NBFC is downgraded below the minimum investment grade, it must immediately stop accepting fresh public deposits and renewing existing deposits [1]. The prohibition on renewing existing deposits applies regardless of whether the NBFC is seeking an upgrade. The NBFC must also regularize excess deposits and report the position to the Reserve Bank within fifteen working days. There is no provision in the passages allowing renewal of existing deposits during the downgrade period or while seeking an upgrade.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3030,7 +3022,7 @@
         </is>
       </c>
       <c r="J48" t="n">
-        <v>6.7</v>
+        <v>5.9</v>
       </c>
       <c r="K48" t="inlineStr"/>
       <c r="L48" t="inlineStr"/>
@@ -3065,12 +3057,12 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Adding a 2% penal interest rate after a missed EMI is permitted, but compounding it is not allowed. Penal charges for non-compliance (e.g., missed EMI) must be treated as separate fees and **not capitalized** (i.e., no further interest computed on such charges) [1][3]. However, normal compounding of interest on unpaid interest (including unpaid EMI) at the contracted rate is allowed until remediation [1]. Thus, the 2% penal interest can be applied, but it cannot be compounded.</t>
+          <t>Adding a 2% penal interest rate after a missed EMI and compounding it is **not permitted**. Penal charges for non-compliance must be treated as separate fees and **cannot be capitalized** (i.e., further interest computed on them). This is explicitly prohibited under the guidelines: "There shall be no capitalisation of penal charges, i.e., no further interest computed on such charges" [1]. Additionally, penal charges must be reasonable, non-discriminatory, and disclosed upfront in the loan agreement [3]. While interest on unpaid interest (including unpaid EMI) may be charged at the contracted rate until remediation, penal charges themselves cannot be compounded.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.12 | 12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.16 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.13 | 12942_Responsible-Business-Conduct.pdf p.35</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.12 | 12942_Responsible-Business-Conduct.pdf p.14 | 12942_Responsible-Business-Conduct.pdf p.16 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.13 | 12942_Responsible-Business-Conduct.pdf p.36</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -3084,7 +3076,7 @@
         </is>
       </c>
       <c r="J49" t="n">
-        <v>7.2</v>
+        <v>7.6</v>
       </c>
       <c r="K49" t="inlineStr"/>
       <c r="L49" t="inlineStr"/>
@@ -3119,12 +3111,12 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Yes, as a Middle Layer NBFC joining an LSP's lending app alongside other lenders, you must report the app to the RBI. According to [1] (18. Reporting of DLAs to RBI), an NBFC must report all DLAs "deployed / joined by them, whether their own or those of the LSPs" on the CIMS portal. This includes participating as a platform participant, even if the app is not owned by the NBFC. The requirement applies regardless of ownership, as the NBFC is actively involved in the arrangement.</t>
+          <t>Yes, you must report the LSP's lending app to the RBI. According to [1] (18. Reporting of DLAs to RBI), an NBFC must report all DLAs "deployed / joined by them, whether their own or those of the LSPs" on the CIMS portal. This includes participation as a platform participant, even if the NBFC does not own the DLA. The requirement applies regardless of ownership, as long as the NBFC is involved in deploying or joining the DLA.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>12957_Credit-Facilities.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12931_Miscellaneous.pdf p.2 | 12957_Credit-Facilities.pdf p.14 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.3 | 12941_Managing-Risks-in-Outsourcing.pdf p.4</t>
+          <t>12957_Credit-Facilities.pdf p.21 | 12953_Concentration-Risk-Management.pdf p.2 | 12931_Miscellaneous.pdf p.2 | 12957_Credit-Facilities.pdf p.15 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12965_Registration-Exemptions-Scale-Based-Regulation.pdf p.20</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -3138,7 +3130,7 @@
         </is>
       </c>
       <c r="J50" t="n">
-        <v>7.2</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="K50" t="inlineStr"/>
       <c r="L50" t="inlineStr"/>
@@ -3173,12 +3165,12 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>No. According to [1], changes in interest rates and charges must be "effected only prospectively," meaning they cannot apply retrospectively. Additionally, [6](8) explicitly prohibits NBFCs from levying charges retrospectively, including pre-payment charges, unless disclosed in advance. Thus, notifying borrowers of a higher contractual rate applying from last month would violate these provisions.</t>
+          <t>No. Changes in interest rates and charges must be effected prospectively, not retrospectively. According to [1], an NBFC shall ensure that changes in interest rates and charges are "effected only prospectively." Additionally, [6] states that pre-payment charges (and by extension, rate changes) must not be applied retrospectively if they were waived earlier. Thus, notifying borrowers of a higher contractual rate applying from last month would violate these rules.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.9 | 12939_Housing-Finance-Companies.pdf p.66 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.36 | 12939_Housing-Finance-Companies.pdf p.101 | 12942_Responsible-Business-Conduct.pdf p.36 | 12942_Responsible-Business-Conduct.pdf p.18</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.9 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.36 | 12939_Housing-Finance-Companies.pdf p.66 | 12939_Housing-Finance-Companies.pdf p.101 | 12942_Responsible-Business-Conduct.pdf p.36 | 12942_Responsible-Business-Conduct.pdf p.18</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -3192,7 +3184,7 @@
         </is>
       </c>
       <c r="J51" t="n">
-        <v>7</v>
+        <v>7.1</v>
       </c>
       <c r="K51" t="inlineStr"/>
       <c r="L51" t="inlineStr"/>
@@ -3226,12 +3218,12 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>The provided context passages do not contain information about SEBI rules governing minimum public shareholding or offer-allocation requirements for NBFCs planning an IPO. The passages focus on RBI regulations related to NBFCs (e.g., sponsorship of IDF-MFs, concentration risk management, and investment guidelines), but none address SEBI's specific requirements for IPOs.</t>
+          <t>The provided context passages do not contain specific information about minimum public shareholding or offer-allocation requirements for NBFCs under SEBI rules for an IPO. The closest reference is to exemptions from SEBI regulations for restructurings under RBI guidelines [6], but this pertains to debt-equity conversions and restructuring, not IPOs. No direct answer is available in the given texts.</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>12931_Miscellaneous.pdf p.17 | 12961_Undertaking-of-Financial-Services.pdf p.25 | 12938_Standalone-Primary-Dealers.pdf p.47 | 12953_Concentration-Risk-Management.pdf p.2 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12953_Concentration-Risk-Management.pdf p.10</t>
+          <t>12931_Miscellaneous.pdf p.17 | 12961_Undertaking-of-Financial-Services.pdf p.25 | 12953_Concentration-Risk-Management.pdf p.2 | 12953_Concentration-Risk-Management.pdf p.10 | 12961_Undertaking-of-Financial-Services.pdf p.13 | 12947_Resolution-of-Stressed-Assets.pdf p.49</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -3245,7 +3237,7 @@
         </is>
       </c>
       <c r="J52" t="n">
-        <v>7.4</v>
+        <v>6.2</v>
       </c>
       <c r="K52" t="inlineStr"/>
       <c r="L52" t="inlineStr"/>
@@ -3279,12 +3271,12 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>The context passages do not specify a stock-exchange disclosure deadline for material events under SEBI LODR regulations. The provided texts mention compliance requirements (e.g., annual reports [1], listing obligations [2], and exemptions [4]) but do not cite a specific deadline for such disclosures.</t>
+          <t>The context passages do not specify a stock-exchange disclosure deadline for material events under SEBI LODR. No exact timeframe or deadline is provided in the referenced documents.</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>12945_Financial-Statements-Presentation-Disclosures.pdf p.37 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.47 | 12953_Concentration-Risk-Management.pdf p.10 | 12947_Resolution-of-Stressed-Assets.pdf p.49 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.10 | 13587_SUP-Supervisory-Returns.pdf p.9</t>
+          <t>12945_Financial-Statements-Presentation-Disclosures.pdf p.37 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.47 | 12953_Concentration-Risk-Management.pdf p.10 | 12947_Resolution-of-Stressed-Assets.pdf p.49 | 13587_SUP-Supervisory-Returns.pdf p.9 | 12950_Investment-Portfolio-Classification-Valuation.pdf p.10</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
@@ -3298,7 +3290,7 @@
         </is>
       </c>
       <c r="J53" t="n">
-        <v>6.1</v>
+        <v>6.5</v>
       </c>
       <c r="K53" t="inlineStr"/>
       <c r="L53" t="inlineStr"/>
@@ -3337,7 +3329,7 @@
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>12949_Asset-Liability-Management.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.2 | 13587_SUP-Supervisory-Returns.pdf p.7 | 13587_SUP-Supervisory-Returns.pdf p.9 | 12939_Housing-Finance-Companies.pdf p.8 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.2</t>
+          <t>12949_Asset-Liability-Management.pdf p.10 | 12953_Concentration-Risk-Management.pdf p.2 | 13587_SUP-Supervisory-Returns.pdf p.9 | 13587_SUP-Supervisory-Returns.pdf p.7 | 12939_Housing-Finance-Companies.pdf p.8 | 12954_Credit-Risk-Management.pdf p.2</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
@@ -3351,7 +3343,7 @@
         </is>
       </c>
       <c r="J54" t="n">
-        <v>5.7</v>
+        <v>5.3</v>
       </c>
       <c r="K54" t="inlineStr"/>
       <c r="L54" t="inlineStr"/>
@@ -3385,7 +3377,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>The context specifies that employees dealing with insurance agency/broking business must possess "the requisite qualification prescribed by IRDA" [1]. However, the passages do not explicitly name specific examinations or training programs required for these qualifications. The focus is on compliance with IRDA regulations rather than detailing particular exams or training courses.</t>
+          <t>The staff must possess the "requisite qualification prescribed by IRDA" to sell insurance as specified persons of a corporate agent [1]. The passages do not specify exact examinations or training programs, only that compliance with IRDA's prescribed qualifications is required.</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -3395,16 +3387,16 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>REVIEW</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>answered a question the corpus should not cover - check for invention</t>
+          <t>correctly declined to answer</t>
         </is>
       </c>
       <c r="J55" t="n">
-        <v>7.8</v>
+        <v>5.3</v>
       </c>
       <c r="K55" t="inlineStr"/>
       <c r="L55" t="inlineStr"/>
@@ -3443,7 +3435,7 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>12961_Undertaking-of-Financial-Services.pdf p.13 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12943_Know-Your-Customer.pdf p.42 | 12949_Asset-Liability-Management.pdf p.10 | 12943_Know-Your-Customer.pdf p.44 | 12943_Know-Your-Customer.pdf p.41</t>
+          <t>12961_Undertaking-of-Financial-Services.pdf p.13 | 12947_Resolution-of-Stressed-Assets.pdf p.15 | 12943_Know-Your-Customer.pdf p.42 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.53 | 12949_Asset-Liability-Management.pdf p.10 | 12943_Know-Your-Customer.pdf p.44</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -3457,7 +3449,7 @@
         </is>
       </c>
       <c r="J56" t="n">
-        <v>5.2</v>
+        <v>5.6</v>
       </c>
       <c r="K56" t="inlineStr"/>
       <c r="L56" t="inlineStr"/>
@@ -3491,12 +3483,12 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>The provided context passages do not specify the GST rate applicable to loan-processing fees or the timing for issuing tax invoices. The only mention of GST relates to penal charges, stating that NBFCs must follow CBIC instructions on its applicability [4]. No details about GST rates or invoicing timelines for loan-processing fees are provided.</t>
+          <t>The context passages do not specify the GST rate applicable to loan-processing fees or the timing for issuing tax invoices. The only mention of GST relates to penal charges, where NBFCs must follow CBIC instructions [1], but no rate or invoicing timeline is provided for loan-processing fees.</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>12942_Responsible-Business-Conduct.pdf p.35 | 12942_Responsible-Business-Conduct.pdf p.35 | 12942_Responsible-Business-Conduct.pdf p.35 | 12942_Responsible-Business-Conduct.pdf p.14 | 12939_Housing-Finance-Companies.pdf p.53 | 12957_Credit-Facilities.pdf p.10</t>
+          <t>12942_Responsible-Business-Conduct.pdf p.14 | 12939_Housing-Finance-Companies.pdf p.53 | 12957_Credit-Facilities.pdf p.10 | 12939_Housing-Finance-Companies.pdf p.66 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.10 | 12956_Credit-Cards-Issuance-and-Conduct.pdf p.13</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -3510,7 +3502,7 @@
         </is>
       </c>
       <c r="J57" t="n">
-        <v>7.3</v>
+        <v>6.3</v>
       </c>
       <c r="K57" t="inlineStr"/>
       <c r="L57" t="inlineStr"/>
@@ -3544,12 +3536,12 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>The provided context passages do not address whether an NBFC can claim an income-tax deduction for provisions created against bad loans. The discussions focus on accounting disclosures, prudential norms, provisioning requirements, and asset classification, but none mention tax treatment or deductibility of provisions.</t>
+          <t>The provided context passages do not address whether an NBFC can claim an income-tax deduction for provisions created against bad loans. The discussions focus on accounting disclosures, prudential norms, and provisioning requirements under RBI guidelines, but none mention tax treatment or deductibility.</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>12945_Financial-Statements-Presentation-Disclosures.pdf p.8 | 12947_Resolution-of-Stressed-Assets.pdf p.42 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.12 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.26 | 12954_Credit-Risk-Management.pdf p.15 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.14</t>
+          <t>12945_Financial-Statements-Presentation-Disclosures.pdf p.8 | 12947_Resolution-of-Stressed-Assets.pdf p.42 | 12952_Transfer-and-Distribution-of-Credit-Risk.pdf p.26 | 12954_Credit-Risk-Management.pdf p.15 | 12948_Income-Recognition-Asset-Classification-Provisioning.pdf p.14 | 12947_Resolution-of-Stressed-Assets.pdf p.11</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -3563,7 +3555,7 @@
         </is>
       </c>
       <c r="J58" t="n">
-        <v>7.1</v>
+        <v>6.9</v>
       </c>
       <c r="K58" t="inlineStr"/>
       <c r="L58" t="inlineStr"/>
@@ -3597,7 +3589,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>The provided context passages do not mention TDS rates or exemption thresholds for interest payments on resident customers' fixed deposits. The documents focus on legal agreements, interest rate sensitivity statements, and deposit management procedures, but none address tax deduction at source (TDS) regulations or tax exemption thresholds. For this query, refer to the Income Tax Act, 1961, or relevant circulars from the Income Tax Department.</t>
+          <t>The provided context passages do not mention TDS (Tax Deducted at Source) rates or exemption thresholds applicable to interest payments on resident customers' fixed deposits. The documents focus on legal agreements, interest rate sensitivity statements, and financial reporting frameworks, but none address tax deduction rules or thresholds for fixed deposit interest. For accurate TDS information, refer to applicable tax laws or official guidelines from the Income Tax Department.</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3616,7 +3608,7 @@
         </is>
       </c>
       <c r="J59" t="n">
-        <v>8.6</v>
+        <v>7</v>
       </c>
       <c r="K59" t="inlineStr"/>
       <c r="L59" t="inlineStr"/>
@@ -3650,12 +3642,12 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>The context passages do not specify the Companies Act filing deadlines for AOC-4 financial statements or MGT-7 annual returns. The provided information addresses timelines for other returns (e.g., DNBS10, Fraud Monitoring Returns) but does not mention AOC-4 or MGT-7 directly [1][4]. For precise deadlines, reference to the Companies Act, 2013, or relevant regulatory guidelines would be required.</t>
+          <t>The provided context passages do not mention specific filing deadlines for AOC-4 financial statements or MGT-7 annual returns under the Companies Act.</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>13587_SUP-Supervisory-Returns.pdf p.11 | 12935_Mortgage-Guarantee-Companies.pdf p.8 | 12939_Housing-Finance-Companies.pdf p.87 | 13587_SUP-Supervisory-Returns.pdf p.12 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.4 | 12958_Acceptance-of-Public-Deposits.pdf p.18</t>
+          <t>13587_SUP-Supervisory-Returns.pdf p.11 | 12939_Housing-Finance-Companies.pdf p.87 | 13587_SUP-Supervisory-Returns.pdf p.12 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.4 | 12958_Acceptance-of-Public-Deposits.pdf p.18 | 12958_Acceptance-of-Public-Deposits.pdf p.28</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -3669,7 +3661,7 @@
         </is>
       </c>
       <c r="J60" t="n">
-        <v>8</v>
+        <v>5.8</v>
       </c>
       <c r="K60" t="inlineStr"/>
       <c r="L60" t="inlineStr"/>
@@ -3703,12 +3695,12 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>The provided context passages do not contain information about calculating CSR (Corporate Social Responsibility) spending obligations under the Companies Act or transferring unspent CSR amounts. The passages focus on definitions related to public deposits, financial regulations, and capital adequacy, but none address CSR requirements or procedures.</t>
+          <t>The provided context passages do not contain information on calculating Companies Act CSR spending obligations or transferring unspent CSR amounts.</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>12958_Acceptance-of-Public-Deposits.pdf p.8 | 12939_Housing-Finance-Companies.pdf p.6 | 12958_Acceptance-of-Public-Deposits.pdf p.39 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.46 | 12949_Asset-Liability-Management.pdf p.40 | 12959_Prudential-Norms-on-Capital-Adequacy.pdf p.53</t>
+          <t>12958_Acceptance-of-Public-Deposits.pdf p.8 | 12939_Housing-Finance-Companies.pdf p.6 | 12958_Acceptance-of-Public-Deposits.pdf p.39 | 12945_Financial-Statements-Presentation-Disclosures.pdf p.46 | 12949_Asset-Liability-Management.pdf p.40 | 12937_Core-Investment-Companies.pdf p.6</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -3722,7 +3714,7 @@
         </is>
       </c>
       <c r="J61" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
       <c r="K61" t="inlineStr"/>
       <c r="L61" t="inlineStr"/>

</xml_diff>